<commit_message>
Add DUID_TYPE labels and secondary sheet lookup for unidentified assets
- generators.py: add second lookup for Ancillary Services and Wholesale
  Demand Response Units sheets; tag all DUIDs with DUID_TYPE column
- analyse.py: fallback STATION_NAME from STATIONID for unregistered DUIDs;
  infer DUID_TYPE=Network Load from NL suffix pattern for remainder
- index.html: Type badge column with colour-coded pills, Type filter dropdown,
  Type included in Excel export
- Rebuilt outputs: 89 previously-blank DUIDs now identified
</commit_message>
<xml_diff>
--- a/outputs/NSW_mlf.xlsx
+++ b/outputs/NSW_mlf.xlsx
@@ -4007,8 +4007,10 @@
           <t>HUNTER1</t>
         </is>
       </c>
-      <c r="B65" s="2" t="n">
-        <v/>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>HUNTER</t>
+        </is>
       </c>
       <c r="C65" s="2" t="n">
         <v/>
@@ -4895,8 +4897,10 @@
           <t>LIDDNL1</t>
         </is>
       </c>
-      <c r="B81" s="2" t="n">
-        <v/>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>LIDDELL</t>
+        </is>
       </c>
       <c r="C81" s="2" t="n">
         <v/>
@@ -5599,8 +5603,10 @@
           <t>MPNL1</t>
         </is>
       </c>
-      <c r="B93" s="2" t="n">
-        <v/>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
       </c>
       <c r="C93" s="2" t="n">
         <v/>
@@ -5903,8 +5909,10 @@
           <t>TUMUT1-2</t>
         </is>
       </c>
-      <c r="B98" s="2" t="n">
-        <v/>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>TUMUT1</t>
+        </is>
       </c>
       <c r="C98" s="2" t="n">
         <v/>
@@ -5959,8 +5967,10 @@
           <t>TUMUT1-3</t>
         </is>
       </c>
-      <c r="B99" s="2" t="n">
-        <v/>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>TUMUT1</t>
+        </is>
       </c>
       <c r="C99" s="2" t="n">
         <v/>
@@ -6015,8 +6025,10 @@
           <t>TUMUT1-1</t>
         </is>
       </c>
-      <c r="B100" s="2" t="n">
-        <v/>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>TUMUT1</t>
+        </is>
       </c>
       <c r="C100" s="2" t="n">
         <v/>
@@ -6071,8 +6083,10 @@
           <t>TUMUT1-4</t>
         </is>
       </c>
-      <c r="B101" s="2" t="n">
-        <v/>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>TUMUT1</t>
+        </is>
       </c>
       <c r="C101" s="2" t="n">
         <v/>
@@ -6127,8 +6141,10 @@
           <t>TUMUT2-3</t>
         </is>
       </c>
-      <c r="B102" s="2" t="n">
-        <v/>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>TUMUT2</t>
+        </is>
       </c>
       <c r="C102" s="2" t="n">
         <v/>
@@ -6183,8 +6199,10 @@
           <t>TUMUT2-1</t>
         </is>
       </c>
-      <c r="B103" s="2" t="n">
-        <v/>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>TUMUT2</t>
+        </is>
       </c>
       <c r="C103" s="2" t="n">
         <v/>
@@ -6239,8 +6257,10 @@
           <t>TUMUT2-2</t>
         </is>
       </c>
-      <c r="B104" s="2" t="n">
-        <v/>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>TUMUT2</t>
+        </is>
       </c>
       <c r="C104" s="2" t="n">
         <v/>
@@ -6295,8 +6315,10 @@
           <t>TUMUT2-4</t>
         </is>
       </c>
-      <c r="B105" s="2" t="n">
-        <v/>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>TUMUT2</t>
+        </is>
       </c>
       <c r="C105" s="2" t="n">
         <v/>
@@ -7021,8 +7043,10 @@
           <t>VPNL1</t>
         </is>
       </c>
-      <c r="B117" s="2" t="n">
-        <v/>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>VP</t>
+        </is>
       </c>
       <c r="C117" s="2" t="n">
         <v/>
@@ -7201,8 +7225,10 @@
           <t>TUMT3NL3</t>
         </is>
       </c>
-      <c r="B120" s="2" t="n">
-        <v/>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>SNOWY1</t>
+        </is>
       </c>
       <c r="C120" s="2" t="n">
         <v/>
@@ -7257,8 +7283,10 @@
           <t>TUMT3NL2</t>
         </is>
       </c>
-      <c r="B121" s="2" t="n">
-        <v/>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>SNOWY1</t>
+        </is>
       </c>
       <c r="C121" s="2" t="n">
         <v/>
@@ -7313,8 +7341,10 @@
           <t>TUMT3NL1</t>
         </is>
       </c>
-      <c r="B122" s="2" t="n">
-        <v/>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>SNOWY1</t>
+        </is>
       </c>
       <c r="C122" s="2" t="n">
         <v/>
@@ -7431,8 +7461,10 @@
           <t>ERNL1</t>
         </is>
       </c>
-      <c r="B124" s="2" t="n">
-        <v/>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>ERARING</t>
+        </is>
       </c>
       <c r="C124" s="2" t="n">
         <v/>
@@ -8447,8 +8479,10 @@
           <t>DG_NSW1</t>
         </is>
       </c>
-      <c r="B141" s="2" t="n">
-        <v/>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>DG_NSW1</t>
+        </is>
       </c>
       <c r="C141" s="2" t="n">
         <v/>
@@ -8503,8 +8537,10 @@
           <t>STGEORG1</t>
         </is>
       </c>
-      <c r="B142" s="2" t="n">
-        <v/>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>STGEORGE</t>
+        </is>
       </c>
       <c r="C142" s="2" t="n">
         <v/>
@@ -8977,8 +9013,10 @@
           <t>GUTHNL1</t>
         </is>
       </c>
-      <c r="B150" s="2" t="n">
-        <v/>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>SNOWY3</t>
+        </is>
       </c>
       <c r="C150" s="2" t="n">
         <v/>
@@ -9033,8 +9071,10 @@
           <t>TUMUT3-3</t>
         </is>
       </c>
-      <c r="B151" s="2" t="n">
-        <v/>
+      <c r="B151" s="2" t="inlineStr">
+        <is>
+          <t>TUMUT3</t>
+        </is>
       </c>
       <c r="C151" s="2" t="n">
         <v/>
@@ -9089,8 +9129,10 @@
           <t>TUMUT3-2</t>
         </is>
       </c>
-      <c r="B152" s="2" t="n">
-        <v/>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>TUMUT3</t>
+        </is>
       </c>
       <c r="C152" s="2" t="n">
         <v/>
@@ -9145,8 +9187,10 @@
           <t>TUMUT3-1</t>
         </is>
       </c>
-      <c r="B153" s="2" t="n">
-        <v/>
+      <c r="B153" s="2" t="inlineStr">
+        <is>
+          <t>TUMUT3</t>
+        </is>
       </c>
       <c r="C153" s="2" t="n">
         <v/>
@@ -9201,8 +9245,10 @@
           <t>TUMUT3-6</t>
         </is>
       </c>
-      <c r="B154" s="2" t="n">
-        <v/>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>TUMUT3</t>
+        </is>
       </c>
       <c r="C154" s="2" t="n">
         <v/>
@@ -9257,8 +9303,10 @@
           <t>TUMUT3-5</t>
         </is>
       </c>
-      <c r="B155" s="2" t="n">
-        <v/>
+      <c r="B155" s="2" t="inlineStr">
+        <is>
+          <t>TUMUT3</t>
+        </is>
       </c>
       <c r="C155" s="2" t="n">
         <v/>
@@ -9313,8 +9361,10 @@
           <t>TUMUT3-4</t>
         </is>
       </c>
-      <c r="B156" s="2" t="n">
-        <v/>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>TUMUT3</t>
+        </is>
       </c>
       <c r="C156" s="2" t="n">
         <v/>
@@ -9369,8 +9419,10 @@
           <t>REDBANK1</t>
         </is>
       </c>
-      <c r="B157" s="2" t="n">
-        <v/>
+      <c r="B157" s="2" t="inlineStr">
+        <is>
+          <t>REDBANK1</t>
+        </is>
       </c>
       <c r="C157" s="2" t="n">
         <v/>
@@ -9399,8 +9451,10 @@
           <t>HEZ</t>
         </is>
       </c>
-      <c r="B158" s="2" t="n">
-        <v/>
+      <c r="B158" s="2" t="inlineStr">
+        <is>
+          <t>HEZ</t>
+        </is>
       </c>
       <c r="C158" s="2" t="n">
         <v/>
@@ -9431,8 +9485,10 @@
           <t>BANKSPT1</t>
         </is>
       </c>
-      <c r="B159" s="2" t="n">
-        <v/>
+      <c r="B159" s="2" t="inlineStr">
+        <is>
+          <t>BANKSPT</t>
+        </is>
       </c>
       <c r="C159" s="2" t="n">
         <v/>
@@ -9465,8 +9521,10 @@
           <t>AWABAREF</t>
         </is>
       </c>
-      <c r="B160" s="2" t="n">
-        <v/>
+      <c r="B160" s="2" t="inlineStr">
+        <is>
+          <t>AWABAREF</t>
+        </is>
       </c>
       <c r="C160" s="2" t="n">
         <v/>
@@ -9501,8 +9559,10 @@
           <t>NINEWIL1</t>
         </is>
       </c>
-      <c r="B161" s="2" t="n">
-        <v/>
+      <c r="B161" s="2" t="inlineStr">
+        <is>
+          <t>NINEWIL</t>
+        </is>
       </c>
       <c r="C161" s="2" t="n">
         <v/>
@@ -9541,8 +9601,10 @@
           <t>WOYWOY1</t>
         </is>
       </c>
-      <c r="B162" s="2" t="n">
-        <v/>
+      <c r="B162" s="2" t="inlineStr">
+        <is>
+          <t>WOYWOY</t>
+        </is>
       </c>
       <c r="C162" s="2" t="n">
         <v/>
@@ -9583,8 +9645,10 @@
           <t>TERALBA</t>
         </is>
       </c>
-      <c r="B163" s="2" t="n">
-        <v/>
+      <c r="B163" s="2" t="inlineStr">
+        <is>
+          <t>TERALBA</t>
+        </is>
       </c>
       <c r="C163" s="2" t="n">
         <v/>
@@ -9625,8 +9689,10 @@
           <t>KINCUM1</t>
         </is>
       </c>
-      <c r="B164" s="2" t="n">
-        <v/>
+      <c r="B164" s="2" t="inlineStr">
+        <is>
+          <t>KINCUMB</t>
+        </is>
       </c>
       <c r="C164" s="2" t="n">
         <v/>
@@ -9667,8 +9733,10 @@
           <t>LD03</t>
         </is>
       </c>
-      <c r="B165" s="2" t="n">
-        <v/>
+      <c r="B165" s="2" t="inlineStr">
+        <is>
+          <t>LIDDELL</t>
+        </is>
       </c>
       <c r="C165" s="2" t="n">
         <v/>
@@ -9709,8 +9777,10 @@
           <t>HVGTS</t>
         </is>
       </c>
-      <c r="B166" s="2" t="n">
-        <v/>
+      <c r="B166" s="2" t="inlineStr">
+        <is>
+          <t>HUNTVGT</t>
+        </is>
       </c>
       <c r="C166" s="2" t="n">
         <v/>
@@ -9751,8 +9821,10 @@
           <t>AGLNOW1</t>
         </is>
       </c>
-      <c r="B167" s="2" t="n">
-        <v/>
+      <c r="B167" s="2" t="inlineStr">
+        <is>
+          <t>AGLNOW1</t>
+        </is>
       </c>
       <c r="C167" s="2" t="n">
         <v/>
@@ -9793,8 +9865,10 @@
           <t>AGLSITA1</t>
         </is>
       </c>
-      <c r="B168" s="2" t="n">
-        <v/>
+      <c r="B168" s="2" t="inlineStr">
+        <is>
+          <t>AGLSITA</t>
+        </is>
       </c>
       <c r="C168" s="2" t="n">
         <v/>
@@ -9833,8 +9907,10 @@
           <t>LD01</t>
         </is>
       </c>
-      <c r="B169" s="2" t="n">
-        <v/>
+      <c r="B169" s="2" t="inlineStr">
+        <is>
+          <t>LIDDELL</t>
+        </is>
       </c>
       <c r="C169" s="2" t="n">
         <v/>
@@ -9877,8 +9953,10 @@
           <t>LD02</t>
         </is>
       </c>
-      <c r="B170" s="2" t="n">
-        <v/>
+      <c r="B170" s="2" t="inlineStr">
+        <is>
+          <t>LIDDELL</t>
+        </is>
       </c>
       <c r="C170" s="2" t="n">
         <v/>
@@ -9921,8 +9999,10 @@
           <t>LD04</t>
         </is>
       </c>
-      <c r="B171" s="2" t="n">
-        <v/>
+      <c r="B171" s="2" t="inlineStr">
+        <is>
+          <t>LIDDELL</t>
+        </is>
       </c>
       <c r="C171" s="2" t="n">
         <v/>
@@ -9965,8 +10045,10 @@
           <t>WALGRVG1</t>
         </is>
       </c>
-      <c r="B172" s="2" t="n">
-        <v/>
+      <c r="B172" s="2" t="inlineStr">
+        <is>
+          <t>WALGBESS</t>
+        </is>
       </c>
       <c r="C172" s="2" t="n">
         <v/>
@@ -10001,8 +10083,10 @@
           <t>DPNTBG1</t>
         </is>
       </c>
-      <c r="B173" s="2" t="n">
-        <v/>
+      <c r="B173" s="2" t="inlineStr">
+        <is>
+          <t>DPNTBESS</t>
+        </is>
       </c>
       <c r="C173" s="2" t="n">
         <v/>
@@ -10035,8 +10119,10 @@
           <t>BHBG1</t>
         </is>
       </c>
-      <c r="B174" s="2" t="n">
-        <v/>
+      <c r="B174" s="2" t="inlineStr">
+        <is>
+          <t>BHBESS</t>
+        </is>
       </c>
       <c r="C174" s="2" t="n">
         <v/>
@@ -10067,8 +10153,10 @@
           <t>MLLFGEF1</t>
         </is>
       </c>
-      <c r="B175" s="2" t="n">
-        <v/>
+      <c r="B175" s="2" t="inlineStr">
+        <is>
+          <t>MLLFGEF</t>
+        </is>
       </c>
       <c r="C175" s="2" t="n">
         <v/>
@@ -10103,8 +10191,10 @@
           <t>QBYNBG1</t>
         </is>
       </c>
-      <c r="B176" s="2" t="n">
-        <v/>
+      <c r="B176" s="2" t="inlineStr">
+        <is>
+          <t>QBYNBESS</t>
+        </is>
       </c>
       <c r="C176" s="2" t="n">
         <v/>
@@ -10137,8 +10227,10 @@
           <t>RESS1G</t>
         </is>
       </c>
-      <c r="B177" s="2" t="n">
-        <v/>
+      <c r="B177" s="2" t="inlineStr">
+        <is>
+          <t>RESS1</t>
+        </is>
       </c>
       <c r="C177" s="2" t="n">
         <v/>
@@ -10171,8 +10263,10 @@
           <t>RIVNBG2</t>
         </is>
       </c>
-      <c r="B178" s="2" t="n">
-        <v/>
+      <c r="B178" s="2" t="inlineStr">
+        <is>
+          <t>RESS2</t>
+        </is>
       </c>
       <c r="C178" s="2" t="n">
         <v/>
@@ -10205,8 +10299,10 @@
           <t>CAPBES1G</t>
         </is>
       </c>
-      <c r="B179" s="2" t="n">
-        <v/>
+      <c r="B179" s="2" t="inlineStr">
+        <is>
+          <t>CBESS</t>
+        </is>
       </c>
       <c r="C179" s="2" t="n">
         <v/>
@@ -10237,8 +10333,10 @@
           <t>WESTCBT1</t>
         </is>
       </c>
-      <c r="B180" s="2" t="n">
-        <v/>
+      <c r="B180" s="2" t="inlineStr">
+        <is>
+          <t>WESTCBT</t>
+        </is>
       </c>
       <c r="C180" s="2" t="n">
         <v/>
@@ -18182,8 +18280,10 @@
           <t>TUMT3NL3</t>
         </is>
       </c>
-      <c r="B36" s="2" t="n">
-        <v/>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>SNOWY1</t>
+        </is>
       </c>
       <c r="C36" s="2" t="n">
         <v/>
@@ -18207,8 +18307,10 @@
           <t>TUMT3NL2</t>
         </is>
       </c>
-      <c r="B37" s="2" t="n">
-        <v/>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>SNOWY1</t>
+        </is>
       </c>
       <c r="C37" s="2" t="n">
         <v/>
@@ -18232,8 +18334,10 @@
           <t>TUMT3NL1</t>
         </is>
       </c>
-      <c r="B38" s="2" t="n">
-        <v/>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>SNOWY1</t>
+        </is>
       </c>
       <c r="C38" s="2" t="n">
         <v/>

</xml_diff>

<commit_message>
Add MMSDM STATION + GENUNITS lookup for historical/deregistered DUIDs
- generators.py: download STATION and GENUNITS tables from MMSDM archive;
  add 445 historical DUIDs as third metadata tier; cache both tables
- analyse.py: enrich STATION_NAME via MMSDM STATION table (proper full names);
  pass station_names Series through build_summary
- main.py: wire up mmsdm_year/month args and station_names to build_summary
- Result: Unknowns drop from 142 → 12; 170 rows get proper station names;
  fuel type and capacity now populated for batteries, hydro, gas, coal units
</commit_message>
<xml_diff>
--- a/outputs/NSW_mlf.xlsx
+++ b/outputs/NSW_mlf.xlsx
@@ -4009,13 +4009,17 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>HUNTER</t>
-        </is>
-      </c>
-      <c r="C65" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D65" s="2" t="inlineStr"/>
+          <t>Hunter Power Station</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Fossil</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>375</v>
+      </c>
       <c r="E65" s="4" t="inlineStr"/>
       <c r="F65" s="4" t="inlineStr"/>
       <c r="G65" s="4" t="inlineStr"/>
@@ -4899,13 +4903,17 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>LIDDELL</t>
-        </is>
-      </c>
-      <c r="C81" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D81" s="2" t="inlineStr"/>
+          <t>Liddell Power Station</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>Fossil</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>25</v>
+      </c>
       <c r="E81" s="4" t="n">
         <v>0.9676</v>
       </c>
@@ -5605,13 +5613,17 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>MP</t>
-        </is>
-      </c>
-      <c r="C93" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D93" s="2" t="inlineStr"/>
+          <t>MT PIPER POWER STATION</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>Fossil</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>25</v>
+      </c>
       <c r="E93" s="4" t="n">
         <v>0.9744</v>
       </c>
@@ -5914,10 +5926,10 @@
           <t>TUMUT1</t>
         </is>
       </c>
-      <c r="C98" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D98" s="2" t="inlineStr"/>
+      <c r="C98" s="2" t="inlineStr"/>
+      <c r="D98" s="3" t="n">
+        <v>82</v>
+      </c>
       <c r="E98" s="4" t="n">
         <v>0.9768</v>
       </c>
@@ -5972,10 +5984,10 @@
           <t>TUMUT1</t>
         </is>
       </c>
-      <c r="C99" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D99" s="2" t="inlineStr"/>
+      <c r="C99" s="2" t="inlineStr"/>
+      <c r="D99" s="3" t="n">
+        <v>82</v>
+      </c>
       <c r="E99" s="4" t="n">
         <v>0.9768</v>
       </c>
@@ -6030,10 +6042,10 @@
           <t>TUMUT1</t>
         </is>
       </c>
-      <c r="C100" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D100" s="2" t="inlineStr"/>
+      <c r="C100" s="2" t="inlineStr"/>
+      <c r="D100" s="3" t="n">
+        <v>82</v>
+      </c>
       <c r="E100" s="4" t="n">
         <v>0.9768</v>
       </c>
@@ -6088,10 +6100,10 @@
           <t>TUMUT1</t>
         </is>
       </c>
-      <c r="C101" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D101" s="2" t="inlineStr"/>
+      <c r="C101" s="2" t="inlineStr"/>
+      <c r="D101" s="3" t="n">
+        <v>82</v>
+      </c>
       <c r="E101" s="4" t="n">
         <v>0.9768</v>
       </c>
@@ -6146,10 +6158,10 @@
           <t>TUMUT2</t>
         </is>
       </c>
-      <c r="C102" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D102" s="2" t="inlineStr"/>
+      <c r="C102" s="2" t="inlineStr"/>
+      <c r="D102" s="3" t="n">
+        <v>72</v>
+      </c>
       <c r="E102" s="4" t="n">
         <v>0.9768</v>
       </c>
@@ -6204,10 +6216,10 @@
           <t>TUMUT2</t>
         </is>
       </c>
-      <c r="C103" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D103" s="2" t="inlineStr"/>
+      <c r="C103" s="2" t="inlineStr"/>
+      <c r="D103" s="3" t="n">
+        <v>72</v>
+      </c>
       <c r="E103" s="4" t="n">
         <v>0.9768</v>
       </c>
@@ -6262,10 +6274,10 @@
           <t>TUMUT2</t>
         </is>
       </c>
-      <c r="C104" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D104" s="2" t="inlineStr"/>
+      <c r="C104" s="2" t="inlineStr"/>
+      <c r="D104" s="3" t="n">
+        <v>72</v>
+      </c>
       <c r="E104" s="4" t="n">
         <v>0.9768</v>
       </c>
@@ -6320,10 +6332,10 @@
           <t>TUMUT2</t>
         </is>
       </c>
-      <c r="C105" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D105" s="2" t="inlineStr"/>
+      <c r="C105" s="2" t="inlineStr"/>
+      <c r="D105" s="3" t="n">
+        <v>72</v>
+      </c>
       <c r="E105" s="4" t="n">
         <v>0.9768</v>
       </c>
@@ -7045,13 +7057,17 @@
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>VP</t>
-        </is>
-      </c>
-      <c r="C117" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D117" s="2" t="inlineStr"/>
+          <t>Vales Point "B" Power Station</t>
+        </is>
+      </c>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>Fossil</t>
+        </is>
+      </c>
+      <c r="D117" s="3" t="n">
+        <v>25</v>
+      </c>
       <c r="E117" s="4" t="n">
         <v>0.9877</v>
       </c>
@@ -7227,13 +7243,17 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>SNOWY1</t>
-        </is>
-      </c>
-      <c r="C120" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D120" s="2" t="inlineStr"/>
+          <t>Tumut 3 Power Station</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>Hydro</t>
+        </is>
+      </c>
+      <c r="D120" s="3" t="n">
+        <v>25</v>
+      </c>
       <c r="E120" s="4" t="n">
         <v>0.991</v>
       </c>
@@ -7285,13 +7305,17 @@
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>SNOWY1</t>
-        </is>
-      </c>
-      <c r="C121" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D121" s="2" t="inlineStr"/>
+          <t>Tumut 3 Power Station</t>
+        </is>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t>Hydro</t>
+        </is>
+      </c>
+      <c r="D121" s="3" t="n">
+        <v>25</v>
+      </c>
       <c r="E121" s="4" t="n">
         <v>0.991</v>
       </c>
@@ -7343,13 +7367,17 @@
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>SNOWY1</t>
-        </is>
-      </c>
-      <c r="C122" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D122" s="2" t="inlineStr"/>
+          <t>Tumut 3 Power Station</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>Hydro</t>
+        </is>
+      </c>
+      <c r="D122" s="3" t="n">
+        <v>25</v>
+      </c>
       <c r="E122" s="4" t="n">
         <v>0.991</v>
       </c>
@@ -7463,13 +7491,17 @@
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>ERARING</t>
-        </is>
-      </c>
-      <c r="C124" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D124" s="2" t="inlineStr"/>
+          <t>ERARING POWER STATION</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>Fossil</t>
+        </is>
+      </c>
+      <c r="D124" s="3" t="n">
+        <v>25</v>
+      </c>
       <c r="E124" s="4" t="n">
         <v>0.9867</v>
       </c>
@@ -8481,13 +8513,13 @@
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>DG_NSW1</t>
-        </is>
-      </c>
-      <c r="C141" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D141" s="2" t="inlineStr"/>
+          <t>NSW1 Dummy Generator</t>
+        </is>
+      </c>
+      <c r="C141" s="2" t="inlineStr"/>
+      <c r="D141" s="3" t="n">
+        <v>3000</v>
+      </c>
       <c r="E141" s="4" t="n">
         <v>1</v>
       </c>
@@ -8539,13 +8571,17 @@
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>STGEORGE</t>
-        </is>
-      </c>
-      <c r="C142" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D142" s="2" t="inlineStr"/>
+          <t>St George Leagues Plant</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>Fossil</t>
+        </is>
+      </c>
+      <c r="D142" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="E142" s="4" t="n">
         <v>1.0059</v>
       </c>
@@ -9015,13 +9051,17 @@
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
-          <t>SNOWY3</t>
-        </is>
-      </c>
-      <c r="C150" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D150" s="2" t="inlineStr"/>
+          <t>Guthega Power Station</t>
+        </is>
+      </c>
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>Hydro</t>
+        </is>
+      </c>
+      <c r="D150" s="3" t="n">
+        <v>25</v>
+      </c>
       <c r="E150" s="4" t="n">
         <v>0.9549</v>
       </c>
@@ -9076,10 +9116,10 @@
           <t>TUMUT3</t>
         </is>
       </c>
-      <c r="C151" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D151" s="2" t="inlineStr"/>
+      <c r="C151" s="2" t="inlineStr"/>
+      <c r="D151" s="3" t="n">
+        <v>250</v>
+      </c>
       <c r="E151" s="4" t="n">
         <v>1.0092</v>
       </c>
@@ -9134,10 +9174,10 @@
           <t>TUMUT3</t>
         </is>
       </c>
-      <c r="C152" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D152" s="2" t="inlineStr"/>
+      <c r="C152" s="2" t="inlineStr"/>
+      <c r="D152" s="3" t="n">
+        <v>250</v>
+      </c>
       <c r="E152" s="4" t="n">
         <v>1.0092</v>
       </c>
@@ -9192,10 +9232,10 @@
           <t>TUMUT3</t>
         </is>
       </c>
-      <c r="C153" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D153" s="2" t="inlineStr"/>
+      <c r="C153" s="2" t="inlineStr"/>
+      <c r="D153" s="3" t="n">
+        <v>250</v>
+      </c>
       <c r="E153" s="4" t="n">
         <v>1.0092</v>
       </c>
@@ -9250,10 +9290,10 @@
           <t>TUMUT3</t>
         </is>
       </c>
-      <c r="C154" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D154" s="2" t="inlineStr"/>
+      <c r="C154" s="2" t="inlineStr"/>
+      <c r="D154" s="3" t="n">
+        <v>250</v>
+      </c>
       <c r="E154" s="4" t="n">
         <v>1.0092</v>
       </c>
@@ -9308,10 +9348,10 @@
           <t>TUMUT3</t>
         </is>
       </c>
-      <c r="C155" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D155" s="2" t="inlineStr"/>
+      <c r="C155" s="2" t="inlineStr"/>
+      <c r="D155" s="3" t="n">
+        <v>250</v>
+      </c>
       <c r="E155" s="4" t="n">
         <v>1.0092</v>
       </c>
@@ -9366,10 +9406,10 @@
           <t>TUMUT3</t>
         </is>
       </c>
-      <c r="C156" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D156" s="2" t="inlineStr"/>
+      <c r="C156" s="2" t="inlineStr"/>
+      <c r="D156" s="3" t="n">
+        <v>250</v>
+      </c>
       <c r="E156" s="4" t="n">
         <v>1.0092</v>
       </c>
@@ -9421,13 +9461,13 @@
       </c>
       <c r="B157" s="2" t="inlineStr">
         <is>
-          <t>REDBANK1</t>
-        </is>
-      </c>
-      <c r="C157" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D157" s="2" t="inlineStr"/>
+          <t>Redbank Power Station</t>
+        </is>
+      </c>
+      <c r="C157" s="2" t="inlineStr"/>
+      <c r="D157" s="3" t="n">
+        <v>150</v>
+      </c>
       <c r="E157" s="4" t="n">
         <v>0.9843</v>
       </c>
@@ -9453,13 +9493,17 @@
       </c>
       <c r="B158" s="2" t="inlineStr">
         <is>
-          <t>HEZ</t>
-        </is>
-      </c>
-      <c r="C158" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D158" s="2" t="inlineStr"/>
+          <t>Hunter Economic Zone Power Station</t>
+        </is>
+      </c>
+      <c r="C158" s="2" t="inlineStr">
+        <is>
+          <t>Fossil</t>
+        </is>
+      </c>
+      <c r="D158" s="3" t="n">
+        <v>29</v>
+      </c>
       <c r="E158" s="4" t="n">
         <v>0.9969</v>
       </c>
@@ -9487,13 +9531,17 @@
       </c>
       <c r="B159" s="2" t="inlineStr">
         <is>
-          <t>BANKSPT</t>
-        </is>
-      </c>
-      <c r="C159" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D159" s="2" t="inlineStr"/>
+          <t>Bankstown Sports Club Plant Units</t>
+        </is>
+      </c>
+      <c r="C159" s="2" t="inlineStr">
+        <is>
+          <t>Fossil</t>
+        </is>
+      </c>
+      <c r="D159" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="E159" s="4" t="n">
         <v>1.0016</v>
       </c>
@@ -9523,13 +9571,17 @@
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
-          <t>AWABAREF</t>
-        </is>
-      </c>
-      <c r="C160" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D160" s="2" t="inlineStr"/>
+          <t>Awaba Power Station</t>
+        </is>
+      </c>
+      <c r="C160" s="2" t="inlineStr">
+        <is>
+          <t>Other Renewable</t>
+        </is>
+      </c>
+      <c r="D160" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="E160" s="4" t="n">
         <v>0.9926</v>
       </c>
@@ -9561,13 +9613,17 @@
       </c>
       <c r="B161" s="2" t="inlineStr">
         <is>
-          <t>NINEWIL</t>
-        </is>
-      </c>
-      <c r="C161" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D161" s="2" t="inlineStr"/>
+          <t>Nine Network Willoughby Plant</t>
+        </is>
+      </c>
+      <c r="C161" s="2" t="inlineStr">
+        <is>
+          <t>Fossil</t>
+        </is>
+      </c>
+      <c r="D161" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="E161" s="4" t="n">
         <v>1.0051</v>
       </c>
@@ -9603,13 +9659,17 @@
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>WOYWOY</t>
-        </is>
-      </c>
-      <c r="C162" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D162" s="2" t="inlineStr"/>
+          <t>Woy Woy Landfill Site</t>
+        </is>
+      </c>
+      <c r="C162" s="2" t="inlineStr">
+        <is>
+          <t>Other Renewable</t>
+        </is>
+      </c>
+      <c r="D162" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="E162" s="4" t="n">
         <v>1.0017</v>
       </c>
@@ -9647,13 +9707,17 @@
       </c>
       <c r="B163" s="2" t="inlineStr">
         <is>
-          <t>TERALBA</t>
-        </is>
-      </c>
-      <c r="C163" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D163" s="2" t="inlineStr"/>
+          <t>TERALBA POWER STATION</t>
+        </is>
+      </c>
+      <c r="C163" s="2" t="inlineStr">
+        <is>
+          <t>Other Renewable</t>
+        </is>
+      </c>
+      <c r="D163" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="E163" s="4" t="n">
         <v>0.9926</v>
       </c>
@@ -9691,13 +9755,17 @@
       </c>
       <c r="B164" s="2" t="inlineStr">
         <is>
-          <t>KINCUMB</t>
-        </is>
-      </c>
-      <c r="C164" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D164" s="2" t="inlineStr"/>
+          <t>Kincumber Landfill Site</t>
+        </is>
+      </c>
+      <c r="C164" s="2" t="inlineStr">
+        <is>
+          <t>Other Renewable</t>
+        </is>
+      </c>
+      <c r="D164" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="E164" s="4" t="n">
         <v>1.0017</v>
       </c>
@@ -9735,13 +9803,17 @@
       </c>
       <c r="B165" s="2" t="inlineStr">
         <is>
-          <t>LIDDELL</t>
-        </is>
-      </c>
-      <c r="C165" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D165" s="2" t="inlineStr"/>
+          <t>Liddell Power Station</t>
+        </is>
+      </c>
+      <c r="C165" s="2" t="inlineStr">
+        <is>
+          <t>Fossil</t>
+        </is>
+      </c>
+      <c r="D165" s="3" t="n">
+        <v>500</v>
+      </c>
       <c r="E165" s="4" t="n">
         <v>0.9676</v>
       </c>
@@ -9779,7 +9851,7 @@
       </c>
       <c r="B166" s="2" t="inlineStr">
         <is>
-          <t>HUNTVGT</t>
+          <t>Hunter Valley Gas Turbine</t>
         </is>
       </c>
       <c r="C166" s="2" t="n">
@@ -9823,13 +9895,17 @@
       </c>
       <c r="B167" s="2" t="inlineStr">
         <is>
-          <t>AGLNOW1</t>
-        </is>
-      </c>
-      <c r="C167" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D167" s="2" t="inlineStr"/>
+          <t>West Nowra Landfill Gas Power Generation Facility</t>
+        </is>
+      </c>
+      <c r="C167" s="2" t="inlineStr">
+        <is>
+          <t>Other Renewable</t>
+        </is>
+      </c>
+      <c r="D167" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="E167" s="4" t="n">
         <v>0.9916</v>
       </c>
@@ -9867,13 +9943,17 @@
       </c>
       <c r="B168" s="2" t="inlineStr">
         <is>
-          <t>AGLSITA</t>
-        </is>
-      </c>
-      <c r="C168" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D168" s="2" t="inlineStr"/>
+          <t>AGL KEMPS CREEK</t>
+        </is>
+      </c>
+      <c r="C168" s="2" t="inlineStr">
+        <is>
+          <t>Other Renewable</t>
+        </is>
+      </c>
+      <c r="D168" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="E168" s="4" t="inlineStr"/>
       <c r="F168" s="4" t="n">
         <v>1.0019</v>
@@ -9909,13 +9989,17 @@
       </c>
       <c r="B169" s="2" t="inlineStr">
         <is>
-          <t>LIDDELL</t>
-        </is>
-      </c>
-      <c r="C169" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D169" s="2" t="inlineStr"/>
+          <t>Liddell Power Station</t>
+        </is>
+      </c>
+      <c r="C169" s="2" t="inlineStr">
+        <is>
+          <t>Fossil</t>
+        </is>
+      </c>
+      <c r="D169" s="3" t="n">
+        <v>500</v>
+      </c>
       <c r="E169" s="4" t="n">
         <v>0.9676</v>
       </c>
@@ -9955,13 +10039,17 @@
       </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
-          <t>LIDDELL</t>
-        </is>
-      </c>
-      <c r="C170" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D170" s="2" t="inlineStr"/>
+          <t>Liddell Power Station</t>
+        </is>
+      </c>
+      <c r="C170" s="2" t="inlineStr">
+        <is>
+          <t>Fossil</t>
+        </is>
+      </c>
+      <c r="D170" s="3" t="n">
+        <v>500</v>
+      </c>
       <c r="E170" s="4" t="n">
         <v>0.9676</v>
       </c>
@@ -10001,13 +10089,17 @@
       </c>
       <c r="B171" s="2" t="inlineStr">
         <is>
-          <t>LIDDELL</t>
-        </is>
-      </c>
-      <c r="C171" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D171" s="2" t="inlineStr"/>
+          <t>Liddell Power Station</t>
+        </is>
+      </c>
+      <c r="C171" s="2" t="inlineStr">
+        <is>
+          <t>Fossil</t>
+        </is>
+      </c>
+      <c r="D171" s="3" t="n">
+        <v>500</v>
+      </c>
       <c r="E171" s="4" t="n">
         <v>0.9676</v>
       </c>
@@ -10047,13 +10139,17 @@
       </c>
       <c r="B172" s="2" t="inlineStr">
         <is>
-          <t>WALGBESS</t>
-        </is>
-      </c>
-      <c r="C172" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D172" s="2" t="inlineStr"/>
+          <t>Wallgrove BESS 1</t>
+        </is>
+      </c>
+      <c r="C172" s="2" t="inlineStr">
+        <is>
+          <t>Battery</t>
+        </is>
+      </c>
+      <c r="D172" s="3" t="n">
+        <v>50</v>
+      </c>
       <c r="E172" s="4" t="inlineStr"/>
       <c r="F172" s="4" t="inlineStr"/>
       <c r="G172" s="4" t="inlineStr"/>
@@ -10085,13 +10181,17 @@
       </c>
       <c r="B173" s="2" t="inlineStr">
         <is>
-          <t>DPNTBESS</t>
-        </is>
-      </c>
-      <c r="C173" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D173" s="2" t="inlineStr"/>
+          <t>Darlington Point Energy Storage System</t>
+        </is>
+      </c>
+      <c r="C173" s="2" t="inlineStr">
+        <is>
+          <t>Battery</t>
+        </is>
+      </c>
+      <c r="D173" s="3" t="n">
+        <v>25</v>
+      </c>
       <c r="E173" s="4" t="inlineStr"/>
       <c r="F173" s="4" t="inlineStr"/>
       <c r="G173" s="4" t="inlineStr"/>
@@ -10121,13 +10221,17 @@
       </c>
       <c r="B174" s="2" t="inlineStr">
         <is>
-          <t>BHBESS</t>
-        </is>
-      </c>
-      <c r="C174" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D174" s="2" t="inlineStr"/>
+          <t>Broken Hill Battery Energy Storage System</t>
+        </is>
+      </c>
+      <c r="C174" s="2" t="inlineStr">
+        <is>
+          <t>Battery</t>
+        </is>
+      </c>
+      <c r="D174" s="3" t="n">
+        <v>66</v>
+      </c>
       <c r="E174" s="4" t="inlineStr"/>
       <c r="F174" s="4" t="inlineStr"/>
       <c r="G174" s="4" t="inlineStr"/>
@@ -10155,13 +10259,17 @@
       </c>
       <c r="B175" s="2" t="inlineStr">
         <is>
-          <t>MLLFGEF</t>
-        </is>
-      </c>
-      <c r="C175" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D175" s="2" t="inlineStr"/>
+          <t>Mugga Lane Landfill Gas To Energy Facility</t>
+        </is>
+      </c>
+      <c r="C175" s="2" t="inlineStr">
+        <is>
+          <t>Other Renewable</t>
+        </is>
+      </c>
+      <c r="D175" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="E175" s="4" t="inlineStr"/>
       <c r="F175" s="4" t="inlineStr"/>
       <c r="G175" s="4" t="inlineStr"/>
@@ -10193,13 +10301,17 @@
       </c>
       <c r="B176" s="2" t="inlineStr">
         <is>
-          <t>QBYNBESS</t>
-        </is>
-      </c>
-      <c r="C176" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D176" s="2" t="inlineStr"/>
+          <t>Queanbeyan BESS</t>
+        </is>
+      </c>
+      <c r="C176" s="2" t="inlineStr">
+        <is>
+          <t>Battery</t>
+        </is>
+      </c>
+      <c r="D176" s="3" t="n">
+        <v>10</v>
+      </c>
       <c r="E176" s="4" t="inlineStr"/>
       <c r="F176" s="4" t="inlineStr"/>
       <c r="G176" s="4" t="inlineStr"/>
@@ -10229,13 +10341,17 @@
       </c>
       <c r="B177" s="2" t="inlineStr">
         <is>
-          <t>RESS1</t>
-        </is>
-      </c>
-      <c r="C177" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D177" s="2" t="inlineStr"/>
+          <t>Riverina BESS 1</t>
+        </is>
+      </c>
+      <c r="C177" s="2" t="inlineStr">
+        <is>
+          <t>Battery</t>
+        </is>
+      </c>
+      <c r="D177" s="3" t="n">
+        <v>80</v>
+      </c>
       <c r="E177" s="4" t="inlineStr"/>
       <c r="F177" s="4" t="inlineStr"/>
       <c r="G177" s="4" t="inlineStr"/>
@@ -10265,13 +10381,17 @@
       </c>
       <c r="B178" s="2" t="inlineStr">
         <is>
-          <t>RESS2</t>
-        </is>
-      </c>
-      <c r="C178" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D178" s="2" t="inlineStr"/>
+          <t>Riverina Energy Storage System 2</t>
+        </is>
+      </c>
+      <c r="C178" s="2" t="inlineStr">
+        <is>
+          <t>Battery</t>
+        </is>
+      </c>
+      <c r="D178" s="3" t="n">
+        <v>65</v>
+      </c>
       <c r="E178" s="4" t="inlineStr"/>
       <c r="F178" s="4" t="inlineStr"/>
       <c r="G178" s="4" t="inlineStr"/>
@@ -10301,13 +10421,17 @@
       </c>
       <c r="B179" s="2" t="inlineStr">
         <is>
-          <t>CBESS</t>
-        </is>
-      </c>
-      <c r="C179" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D179" s="2" t="inlineStr"/>
+          <t>Capital Battery</t>
+        </is>
+      </c>
+      <c r="C179" s="2" t="inlineStr">
+        <is>
+          <t>Battery</t>
+        </is>
+      </c>
+      <c r="D179" s="3" t="n">
+        <v>125</v>
+      </c>
       <c r="E179" s="4" t="inlineStr"/>
       <c r="F179" s="4" t="inlineStr"/>
       <c r="G179" s="4" t="inlineStr"/>
@@ -10335,13 +10459,17 @@
       </c>
       <c r="B180" s="2" t="inlineStr">
         <is>
-          <t>WESTCBT</t>
-        </is>
-      </c>
-      <c r="C180" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D180" s="2" t="inlineStr"/>
+          <t>Western Suburbs League Club (Campbelltown) Plant</t>
+        </is>
+      </c>
+      <c r="C180" s="2" t="inlineStr">
+        <is>
+          <t>Fossil</t>
+        </is>
+      </c>
+      <c r="D180" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="E180" s="4" t="n">
         <v>0.9991</v>
       </c>
@@ -18282,11 +18410,13 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>SNOWY1</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="n">
-        <v/>
+          <t>Tumut 3 Power Station</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Hydro</t>
+        </is>
       </c>
       <c r="D36" s="4" t="n">
         <v>0.9887</v>
@@ -18309,11 +18439,13 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>SNOWY1</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="n">
-        <v/>
+          <t>Tumut 3 Power Station</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Hydro</t>
+        </is>
       </c>
       <c r="D37" s="4" t="n">
         <v>0.9887</v>
@@ -18336,11 +18468,13 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>SNOWY1</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="n">
-        <v/>
+          <t>Tumut 3 Power Station</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Hydro</t>
+        </is>
       </c>
       <c r="D38" s="4" t="n">
         <v>0.9887</v>

</xml_diff>

<commit_message>
Update MLF data 2026-05-11
</commit_message>
<xml_diff>
--- a/outputs/NSW_mlf.xlsx
+++ b/outputs/NSW_mlf.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MLF Table" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Biggest Movers" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="MLF Table" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Heatmap" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Biggest Movers" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -725,27 +725,25 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>WRWF1</t>
+          <t>WRSF1</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>White Rock Wind Farm</t>
+          <t>White Rock Solar Farm</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Wind</t>
+          <t>Solar</t>
         </is>
       </c>
       <c r="D4" s="4" t="n">
-        <v>175</v>
+        <v>22</v>
       </c>
       <c r="E4" s="5" t="inlineStr"/>
       <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="n">
-        <v>0.8468</v>
-      </c>
+      <c r="G4" s="5" t="inlineStr"/>
       <c r="H4" s="5" t="n">
         <v>0.8427</v>
       </c>
@@ -788,25 +786,27 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>WRSF1</t>
+          <t>WRWF1</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>White Rock Solar Farm</t>
+          <t>White Rock Wind Farm</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Solar</t>
+          <t>Wind</t>
         </is>
       </c>
       <c r="D5" s="4" t="n">
-        <v>22</v>
+        <v>175</v>
       </c>
       <c r="E5" s="5" t="inlineStr"/>
       <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="n">
+        <v>0.8468</v>
+      </c>
       <c r="H5" s="5" t="n">
         <v>0.8427</v>
       </c>
@@ -1860,12 +1860,12 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>WYASF1</t>
+          <t>WSTWYSF1</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Wyalong Solar Farm</t>
+          <t>West Wyalong Solar Farm</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -1874,7 +1874,7 @@
         </is>
       </c>
       <c r="D23" s="4" t="n">
-        <v>62</v>
+        <v>105</v>
       </c>
       <c r="E23" s="5" t="inlineStr"/>
       <c r="F23" s="5" t="inlineStr"/>
@@ -1913,12 +1913,12 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>WSTWYSF1</t>
+          <t>WYASF1</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>West Wyalong Solar Farm</t>
+          <t>Wyalong Solar Farm</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -1927,7 +1927,7 @@
         </is>
       </c>
       <c r="D24" s="4" t="n">
-        <v>105</v>
+        <v>62</v>
       </c>
       <c r="E24" s="5" t="inlineStr"/>
       <c r="F24" s="5" t="inlineStr"/>
@@ -2170,7 +2170,7 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>NEWENSF2</t>
+          <t>NEWENSF1</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -2223,7 +2223,7 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>NEWENSF1</t>
+          <t>NEWENSF2</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -2276,12 +2276,12 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>GOONSF1</t>
+          <t>PARSF1</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Goonumbla Solar Farm</t>
+          <t>Parkes Solar Farm</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -2290,14 +2290,18 @@
         </is>
       </c>
       <c r="D31" s="4" t="n">
-        <v>85</v>
+        <v>55</v>
       </c>
       <c r="E31" s="5" t="inlineStr"/>
       <c r="F31" s="5" t="inlineStr"/>
-      <c r="G31" s="5" t="inlineStr"/>
-      <c r="H31" s="5" t="inlineStr"/>
+      <c r="G31" s="5" t="n">
+        <v>1.0135</v>
+      </c>
+      <c r="H31" s="5" t="n">
+        <v>0.9964</v>
+      </c>
       <c r="I31" s="5" t="n">
-        <v>0.9791</v>
+        <v>0.9812</v>
       </c>
       <c r="J31" s="5" t="n">
         <v>0.9258999999999999</v>
@@ -2335,12 +2339,12 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>PARSF1</t>
+          <t>GOONSF1</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Parkes Solar Farm</t>
+          <t>Goonumbla Solar Farm</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -2349,18 +2353,14 @@
         </is>
       </c>
       <c r="D32" s="4" t="n">
-        <v>55</v>
+        <v>85</v>
       </c>
       <c r="E32" s="5" t="inlineStr"/>
       <c r="F32" s="5" t="inlineStr"/>
-      <c r="G32" s="5" t="n">
-        <v>1.0135</v>
-      </c>
-      <c r="H32" s="5" t="n">
-        <v>0.9964</v>
-      </c>
+      <c r="G32" s="5" t="inlineStr"/>
+      <c r="H32" s="5" t="inlineStr"/>
       <c r="I32" s="5" t="n">
-        <v>0.9812</v>
+        <v>0.9791</v>
       </c>
       <c r="J32" s="5" t="n">
         <v>0.9258999999999999</v>
@@ -2632,7 +2632,7 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>QPSFB2</t>
+          <t>QPSFB1</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -2642,11 +2642,11 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Battery</t>
+          <t>Solar</t>
         </is>
       </c>
       <c r="D37" s="4" t="n">
-        <v>27</v>
+        <v>96</v>
       </c>
       <c r="E37" s="5" t="inlineStr"/>
       <c r="F37" s="5" t="inlineStr"/>
@@ -2668,26 +2668,20 @@
       <c r="R37" s="5" t="n">
         <v>0.9032</v>
       </c>
-      <c r="S37" s="5" t="n">
-        <v>0.9032</v>
-      </c>
+      <c r="S37" s="5" t="inlineStr"/>
       <c r="T37" s="5" t="n">
         <v>-0.1158</v>
       </c>
       <c r="U37" s="6" t="n">
         <v>-11.36</v>
       </c>
-      <c r="V37" s="5" t="n">
-        <v>-0.0144</v>
-      </c>
-      <c r="W37" s="6" t="n">
-        <v>-1.57</v>
-      </c>
+      <c r="V37" s="5" t="inlineStr"/>
+      <c r="W37" s="6" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>QPSFB1</t>
+          <t>QPSFB2</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -2697,11 +2691,11 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Solar</t>
+          <t>Battery</t>
         </is>
       </c>
       <c r="D38" s="4" t="n">
-        <v>96</v>
+        <v>27</v>
       </c>
       <c r="E38" s="5" t="inlineStr"/>
       <c r="F38" s="5" t="inlineStr"/>
@@ -2723,15 +2717,21 @@
       <c r="R38" s="5" t="n">
         <v>0.9032</v>
       </c>
-      <c r="S38" s="5" t="inlineStr"/>
+      <c r="S38" s="5" t="n">
+        <v>0.9032</v>
+      </c>
       <c r="T38" s="5" t="n">
         <v>-0.1158</v>
       </c>
       <c r="U38" s="6" t="n">
         <v>-11.36</v>
       </c>
-      <c r="V38" s="5" t="inlineStr"/>
-      <c r="W38" s="6" t="inlineStr"/>
+      <c r="V38" s="5" t="n">
+        <v>-0.0144</v>
+      </c>
+      <c r="W38" s="6" t="n">
+        <v>-1.57</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -2968,7 +2968,7 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>URANQ13</t>
+          <t>URANQ14</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -3169,7 +3169,7 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>URANQ14</t>
+          <t>URANQ13</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -3354,51 +3354,55 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>SKSF1</t>
+          <t>GUTHEGA</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>South Keswick Solar Farm</t>
+          <t>Guthega Power Station</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Solar</t>
+          <t>Hydro</t>
         </is>
       </c>
       <c r="D49" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="E49" s="5" t="inlineStr"/>
-      <c r="F49" s="5" t="inlineStr"/>
+        <v>60</v>
+      </c>
+      <c r="E49" s="5" t="n">
+        <v>0.8882</v>
+      </c>
+      <c r="F49" s="5" t="n">
+        <v>0.9371</v>
+      </c>
       <c r="G49" s="5" t="n">
-        <v>0.9714</v>
+        <v>0.9658</v>
       </c>
       <c r="H49" s="5" t="n">
-        <v>0.9708</v>
+        <v>0.9537</v>
       </c>
       <c r="I49" s="5" t="n">
-        <v>0.9603</v>
+        <v>0.9016</v>
       </c>
       <c r="J49" s="5" t="n">
-        <v>0.9569</v>
+        <v>0.9125</v>
       </c>
       <c r="K49" s="5" t="n">
-        <v>0.9444</v>
+        <v>0.9006</v>
       </c>
       <c r="L49" s="5" t="n">
-        <v>0.9352</v>
+        <v>0.887</v>
       </c>
       <c r="M49" s="5" t="n">
-        <v>0.9439</v>
+        <v>0.893</v>
       </c>
       <c r="N49" s="5" t="n">
-        <v>0.9284</v>
+        <v>0.892</v>
       </c>
       <c r="O49" s="5" t="inlineStr"/>
       <c r="P49" s="5" t="n">
-        <v>0.923</v>
+        <v>0.9135</v>
       </c>
       <c r="Q49" s="5" t="inlineStr"/>
       <c r="R49" s="5" t="n">
@@ -3406,10 +3410,10 @@
       </c>
       <c r="S49" s="5" t="inlineStr"/>
       <c r="T49" s="5" t="n">
-        <v>0.0043</v>
+        <v>0.0138</v>
       </c>
       <c r="U49" s="6" t="n">
-        <v>0.47</v>
+        <v>1.51</v>
       </c>
       <c r="V49" s="5" t="inlineStr"/>
       <c r="W49" s="6" t="inlineStr"/>
@@ -3417,12 +3421,12 @@
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>NEVERSF1</t>
+          <t>SKSF1</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>Nevertire Solar Farm</t>
+          <t>South Keswick Solar Farm</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
@@ -3431,14 +3435,18 @@
         </is>
       </c>
       <c r="D50" s="4" t="n">
-        <v>132</v>
+        <v>15</v>
       </c>
       <c r="E50" s="5" t="inlineStr"/>
       <c r="F50" s="5" t="inlineStr"/>
-      <c r="G50" s="5" t="inlineStr"/>
-      <c r="H50" s="5" t="inlineStr"/>
+      <c r="G50" s="5" t="n">
+        <v>0.9714</v>
+      </c>
+      <c r="H50" s="5" t="n">
+        <v>0.9708</v>
+      </c>
       <c r="I50" s="5" t="n">
-        <v>0.9582000000000001</v>
+        <v>0.9603</v>
       </c>
       <c r="J50" s="5" t="n">
         <v>0.9569</v>
@@ -3476,12 +3484,12 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>NASF1</t>
+          <t>WELLSF1</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Narromine Solar Farm</t>
+          <t xml:space="preserve">Wellington Solar Farm </t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
@@ -3490,21 +3498,15 @@
         </is>
       </c>
       <c r="D51" s="4" t="n">
-        <v>10</v>
+        <v>216</v>
       </c>
       <c r="E51" s="5" t="inlineStr"/>
       <c r="F51" s="5" t="inlineStr"/>
-      <c r="G51" s="5" t="n">
-        <v>0.9714</v>
-      </c>
-      <c r="H51" s="5" t="n">
-        <v>0.9708</v>
-      </c>
-      <c r="I51" s="5" t="n">
-        <v>0.9603</v>
-      </c>
+      <c r="G51" s="5" t="inlineStr"/>
+      <c r="H51" s="5" t="inlineStr"/>
+      <c r="I51" s="5" t="inlineStr"/>
       <c r="J51" s="5" t="n">
-        <v>0.9569</v>
+        <v>0.9471000000000001</v>
       </c>
       <c r="K51" s="5" t="n">
         <v>0.9444</v>
@@ -3539,12 +3541,12 @@
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>WELLSF1</t>
+          <t>NEVERSF1</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wellington Solar Farm </t>
+          <t>Nevertire Solar Farm</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
@@ -3553,15 +3555,17 @@
         </is>
       </c>
       <c r="D52" s="4" t="n">
-        <v>216</v>
+        <v>132</v>
       </c>
       <c r="E52" s="5" t="inlineStr"/>
       <c r="F52" s="5" t="inlineStr"/>
       <c r="G52" s="5" t="inlineStr"/>
       <c r="H52" s="5" t="inlineStr"/>
-      <c r="I52" s="5" t="inlineStr"/>
+      <c r="I52" s="5" t="n">
+        <v>0.9582000000000001</v>
+      </c>
       <c r="J52" s="5" t="n">
-        <v>0.9471000000000001</v>
+        <v>0.9569</v>
       </c>
       <c r="K52" s="5" t="n">
         <v>0.9444</v>
@@ -3596,55 +3600,51 @@
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>GUTHEGA</t>
+          <t>NASF1</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>Guthega Power Station</t>
+          <t>Narromine Solar Farm</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Hydro</t>
+          <t>Solar</t>
         </is>
       </c>
       <c r="D53" s="4" t="n">
-        <v>60</v>
-      </c>
-      <c r="E53" s="5" t="n">
-        <v>0.8882</v>
-      </c>
-      <c r="F53" s="5" t="n">
-        <v>0.9371</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="E53" s="5" t="inlineStr"/>
+      <c r="F53" s="5" t="inlineStr"/>
       <c r="G53" s="5" t="n">
-        <v>0.9658</v>
+        <v>0.9714</v>
       </c>
       <c r="H53" s="5" t="n">
-        <v>0.9537</v>
+        <v>0.9708</v>
       </c>
       <c r="I53" s="5" t="n">
-        <v>0.9016</v>
+        <v>0.9603</v>
       </c>
       <c r="J53" s="5" t="n">
-        <v>0.9125</v>
+        <v>0.9569</v>
       </c>
       <c r="K53" s="5" t="n">
-        <v>0.9006</v>
+        <v>0.9444</v>
       </c>
       <c r="L53" s="5" t="n">
-        <v>0.887</v>
+        <v>0.9352</v>
       </c>
       <c r="M53" s="5" t="n">
-        <v>0.893</v>
+        <v>0.9439</v>
       </c>
       <c r="N53" s="5" t="n">
-        <v>0.892</v>
+        <v>0.9284</v>
       </c>
       <c r="O53" s="5" t="inlineStr"/>
       <c r="P53" s="5" t="n">
-        <v>0.9135</v>
+        <v>0.923</v>
       </c>
       <c r="Q53" s="5" t="inlineStr"/>
       <c r="R53" s="5" t="n">
@@ -3652,10 +3652,10 @@
       </c>
       <c r="S53" s="5" t="inlineStr"/>
       <c r="T53" s="5" t="n">
-        <v>0.0138</v>
+        <v>0.0043</v>
       </c>
       <c r="U53" s="6" t="n">
-        <v>1.51</v>
+        <v>0.47</v>
       </c>
       <c r="V53" s="5" t="inlineStr"/>
       <c r="W53" s="6" t="inlineStr"/>
@@ -4446,12 +4446,12 @@
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>CULLRGWF</t>
+          <t>GUNNING1</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>Cullerin Range Wind Farm</t>
+          <t>Gunning Wind Farm</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
@@ -4460,7 +4460,7 @@
         </is>
       </c>
       <c r="D67" s="4" t="n">
-        <v>30</v>
+        <v>46.5</v>
       </c>
       <c r="E67" s="5" t="n">
         <v>0.9742</v>
@@ -4513,12 +4513,12 @@
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>GUNNING1</t>
+          <t>CULLRGWF</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>Gunning Wind Farm</t>
+          <t>Cullerin Range Wind Farm</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
@@ -4527,7 +4527,7 @@
         </is>
       </c>
       <c r="D68" s="4" t="n">
-        <v>46.5</v>
+        <v>30</v>
       </c>
       <c r="E68" s="5" t="n">
         <v>0.9742</v>
@@ -4621,7 +4621,7 @@
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>HUNTER2</t>
+          <t>HUNTER1</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
@@ -4670,7 +4670,7 @@
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>HUNTER1</t>
+          <t>HUNTER2</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
@@ -6075,12 +6075,12 @@
     <row r="94">
       <c r="A94" s="3" t="inlineStr">
         <is>
-          <t>WOODLWN1</t>
+          <t>CAPTL_WF</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>Woodlawn Wind Farm</t>
+          <t>Capital Wind Farm</t>
         </is>
       </c>
       <c r="C94" s="3" t="inlineStr">
@@ -6089,7 +6089,7 @@
         </is>
       </c>
       <c r="D94" s="4" t="n">
-        <v>48.3</v>
+        <v>140</v>
       </c>
       <c r="E94" s="5" t="n">
         <v>0.9748</v>
@@ -6142,12 +6142,12 @@
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>CAPTL_WF</t>
+          <t>WOODLWN1</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>Capital Wind Farm</t>
+          <t>Woodlawn Wind Farm</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
@@ -6156,7 +6156,7 @@
         </is>
       </c>
       <c r="D95" s="4" t="n">
-        <v>140</v>
+        <v>48.3</v>
       </c>
       <c r="E95" s="5" t="n">
         <v>0.9748</v>
@@ -6276,21 +6276,21 @@
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t>NYNGAN1</t>
+          <t>BDONGHYD</t>
         </is>
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>Nyngan Solar Plant</t>
+          <t>Burrendong Hydro Power Station</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>Solar</t>
+          <t>Hydro</t>
         </is>
       </c>
       <c r="D97" s="4" t="n">
-        <v>102.141</v>
+        <v>19</v>
       </c>
       <c r="E97" s="5" t="n">
         <v>0.9903</v>
@@ -6343,21 +6343,21 @@
     <row r="98">
       <c r="A98" s="3" t="inlineStr">
         <is>
-          <t>BDONGHYD</t>
+          <t>NYNGAN1</t>
         </is>
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>Burrendong Hydro Power Station</t>
+          <t>Nyngan Solar Plant</t>
         </is>
       </c>
       <c r="C98" s="3" t="inlineStr">
         <is>
-          <t>Hydro</t>
+          <t>Solar</t>
         </is>
       </c>
       <c r="D98" s="4" t="n">
-        <v>19</v>
+        <v>102.141</v>
       </c>
       <c r="E98" s="5" t="n">
         <v>0.9903</v>
@@ -6542,7 +6542,7 @@
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>MP2</t>
+          <t>MP1</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
@@ -6609,7 +6609,7 @@
     <row r="102">
       <c r="A102" s="3" t="inlineStr">
         <is>
-          <t>MP1</t>
+          <t>MP2</t>
         </is>
       </c>
       <c r="B102" s="3" t="inlineStr">
@@ -6676,21 +6676,21 @@
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>GLBWNHYD</t>
+          <t>GLENNCRK</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>Glenbawn Hydro Power Station</t>
+          <t>Glennies Creek Power Station</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
         <is>
-          <t>Hydro</t>
+          <t>Fossil</t>
         </is>
       </c>
       <c r="D103" s="4" t="n">
-        <v>5.5</v>
+        <v>12.78</v>
       </c>
       <c r="E103" s="5" t="n">
         <v>0.9828</v>
@@ -6743,21 +6743,21 @@
     <row r="104">
       <c r="A104" s="3" t="inlineStr">
         <is>
-          <t>GLENNCRK</t>
+          <t>GLBWNHYD</t>
         </is>
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>Glennies Creek Power Station</t>
+          <t>Glenbawn Hydro Power Station</t>
         </is>
       </c>
       <c r="C104" s="3" t="inlineStr">
         <is>
-          <t>Fossil</t>
+          <t>Hydro</t>
         </is>
       </c>
       <c r="D104" s="4" t="n">
-        <v>12.78</v>
+        <v>5.5</v>
       </c>
       <c r="E104" s="5" t="n">
         <v>0.9828</v>
@@ -6869,17 +6869,17 @@
     <row r="106">
       <c r="A106" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1-1</t>
+          <t>TUMUT2-4</t>
         </is>
       </c>
       <c r="B106" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1</t>
+          <t>TUMUT2</t>
         </is>
       </c>
       <c r="C106" s="3" t="inlineStr"/>
       <c r="D106" s="4" t="n">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="E106" s="5" t="n">
         <v>0.9768</v>
@@ -6932,17 +6932,17 @@
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1-2</t>
+          <t>TUMUT2-1</t>
         </is>
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1</t>
+          <t>TUMUT2</t>
         </is>
       </c>
       <c r="C107" s="3" t="inlineStr"/>
       <c r="D107" s="4" t="n">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="E107" s="5" t="n">
         <v>0.9768</v>
@@ -6995,7 +6995,7 @@
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1-3</t>
+          <t>TUMUT1-4</t>
         </is>
       </c>
       <c r="B108" s="3" t="inlineStr">
@@ -7058,7 +7058,7 @@
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2-4</t>
+          <t>TUMUT2-3</t>
         </is>
       </c>
       <c r="B109" s="3" t="inlineStr">
@@ -7184,17 +7184,17 @@
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2-1</t>
+          <t>TUMUT1-3</t>
         </is>
       </c>
       <c r="B111" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2</t>
+          <t>TUMUT1</t>
         </is>
       </c>
       <c r="C111" s="3" t="inlineStr"/>
       <c r="D111" s="4" t="n">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="E111" s="5" t="n">
         <v>0.9768</v>
@@ -7247,7 +7247,7 @@
     <row r="112">
       <c r="A112" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1-4</t>
+          <t>TUMUT1-1</t>
         </is>
       </c>
       <c r="B112" s="3" t="inlineStr">
@@ -7310,17 +7310,17 @@
     <row r="113">
       <c r="A113" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2-3</t>
+          <t>TUMUT1-2</t>
         </is>
       </c>
       <c r="B113" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2</t>
+          <t>TUMUT1</t>
         </is>
       </c>
       <c r="C113" s="3" t="inlineStr"/>
       <c r="D113" s="4" t="n">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="E113" s="5" t="n">
         <v>0.9768</v>
@@ -7499,8 +7499,14 @@
           <t>Eraring Battery Energy Storage System</t>
         </is>
       </c>
-      <c r="C116" s="3" t="n"/>
-      <c r="D116" s="3" t="inlineStr"/>
+      <c r="C116" s="3" t="inlineStr">
+        <is>
+          <t>Battery</t>
+        </is>
+      </c>
+      <c r="D116" s="4" t="n">
+        <v>614.6</v>
+      </c>
       <c r="E116" s="5" t="inlineStr"/>
       <c r="F116" s="5" t="inlineStr"/>
       <c r="G116" s="5" t="inlineStr"/>
@@ -7544,7 +7550,7 @@
     <row r="117">
       <c r="A117" s="3" t="inlineStr">
         <is>
-          <t>CG3</t>
+          <t>CG1</t>
         </is>
       </c>
       <c r="B117" s="3" t="inlineStr">
@@ -7611,7 +7617,7 @@
     <row r="118">
       <c r="A118" s="3" t="inlineStr">
         <is>
-          <t>CG2</t>
+          <t>CG3</t>
         </is>
       </c>
       <c r="B118" s="3" t="inlineStr">
@@ -7678,7 +7684,7 @@
     <row r="119">
       <c r="A119" s="3" t="inlineStr">
         <is>
-          <t>CG4</t>
+          <t>CG2</t>
         </is>
       </c>
       <c r="B119" s="3" t="inlineStr">
@@ -7745,7 +7751,7 @@
     <row r="120">
       <c r="A120" s="3" t="inlineStr">
         <is>
-          <t>CG1</t>
+          <t>CG4</t>
         </is>
       </c>
       <c r="B120" s="3" t="inlineStr">
@@ -7871,7 +7877,7 @@
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
         <is>
-          <t>ERGT01</t>
+          <t>ER01</t>
         </is>
       </c>
       <c r="B122" s="3" t="inlineStr">
@@ -7885,7 +7891,7 @@
         </is>
       </c>
       <c r="D122" s="4" t="n">
-        <v>41.5</v>
+        <v>720</v>
       </c>
       <c r="E122" s="5" t="n">
         <v>0.9856</v>
@@ -7938,7 +7944,7 @@
     <row r="123">
       <c r="A123" s="3" t="inlineStr">
         <is>
-          <t>ER02</t>
+          <t>ERGT01</t>
         </is>
       </c>
       <c r="B123" s="3" t="inlineStr">
@@ -7952,7 +7958,7 @@
         </is>
       </c>
       <c r="D123" s="4" t="n">
-        <v>720</v>
+        <v>41.5</v>
       </c>
       <c r="E123" s="5" t="n">
         <v>0.9856</v>
@@ -8005,7 +8011,7 @@
     <row r="124">
       <c r="A124" s="3" t="inlineStr">
         <is>
-          <t>ER01</t>
+          <t>ER02</t>
         </is>
       </c>
       <c r="B124" s="3" t="inlineStr">
@@ -8446,7 +8452,7 @@
     <row r="131">
       <c r="A131" s="3" t="inlineStr">
         <is>
-          <t>VP6</t>
+          <t>VP5</t>
         </is>
       </c>
       <c r="B131" s="3" t="inlineStr">
@@ -8513,7 +8519,7 @@
     <row r="132">
       <c r="A132" s="3" t="inlineStr">
         <is>
-          <t>VPNL1</t>
+          <t>VP6</t>
         </is>
       </c>
       <c r="B132" s="3" t="inlineStr">
@@ -8527,7 +8533,7 @@
         </is>
       </c>
       <c r="D132" s="4" t="n">
-        <v>25</v>
+        <v>660</v>
       </c>
       <c r="E132" s="5" t="n">
         <v>0.9877</v>
@@ -8580,7 +8586,7 @@
     <row r="133">
       <c r="A133" s="3" t="inlineStr">
         <is>
-          <t>VP5</t>
+          <t>VPNL1</t>
         </is>
       </c>
       <c r="B133" s="3" t="inlineStr">
@@ -8594,7 +8600,7 @@
         </is>
       </c>
       <c r="D133" s="4" t="n">
-        <v>660</v>
+        <v>25</v>
       </c>
       <c r="E133" s="5" t="n">
         <v>0.9877</v>
@@ -8714,7 +8720,7 @@
     <row r="135">
       <c r="A135" s="3" t="inlineStr">
         <is>
-          <t>TUMT3NL1</t>
+          <t>TUMT3NL2</t>
         </is>
       </c>
       <c r="B135" s="3" t="inlineStr">
@@ -8781,7 +8787,7 @@
     <row r="136">
       <c r="A136" s="3" t="inlineStr">
         <is>
-          <t>TUMT3NL2</t>
+          <t>TUMT3NL3</t>
         </is>
       </c>
       <c r="B136" s="3" t="inlineStr">
@@ -8848,7 +8854,7 @@
     <row r="137">
       <c r="A137" s="3" t="inlineStr">
         <is>
-          <t>TUMT3NL3</t>
+          <t>TUMT3NL1</t>
         </is>
       </c>
       <c r="B137" s="3" t="inlineStr">
@@ -9653,12 +9659,12 @@
     <row r="150">
       <c r="A150" s="3" t="inlineStr">
         <is>
-          <t>WYANGALB</t>
+          <t>WYANGALA</t>
         </is>
       </c>
       <c r="B150" s="3" t="inlineStr">
         <is>
-          <t>Wyangala B Power Station</t>
+          <t>Wyangala A Power Station</t>
         </is>
       </c>
       <c r="C150" s="3" t="inlineStr">
@@ -9667,7 +9673,7 @@
         </is>
       </c>
       <c r="D150" s="4" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="E150" s="5" t="n">
         <v>1.0099</v>
@@ -9720,12 +9726,12 @@
     <row r="151">
       <c r="A151" s="3" t="inlineStr">
         <is>
-          <t>WYANGALA</t>
+          <t>WYANGALB</t>
         </is>
       </c>
       <c r="B151" s="3" t="inlineStr">
         <is>
-          <t>Wyangala A Power Station</t>
+          <t>Wyangala B Power Station</t>
         </is>
       </c>
       <c r="C151" s="3" t="inlineStr">
@@ -9734,7 +9740,7 @@
         </is>
       </c>
       <c r="D151" s="4" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="E151" s="5" t="n">
         <v>1.0099</v>
@@ -9787,7 +9793,7 @@
     <row r="152">
       <c r="A152" s="3" t="inlineStr">
         <is>
-          <t>LUCAS2S2</t>
+          <t>LUCASHGT</t>
         </is>
       </c>
       <c r="B152" s="3" t="inlineStr">
@@ -9801,7 +9807,7 @@
         </is>
       </c>
       <c r="D152" s="4" t="n">
-        <v>4.6</v>
+        <v>12.65</v>
       </c>
       <c r="E152" s="5" t="n">
         <v>1.0016</v>
@@ -9854,7 +9860,7 @@
     <row r="153">
       <c r="A153" s="3" t="inlineStr">
         <is>
-          <t>LUCASHGT</t>
+          <t>LUCAS2S2</t>
         </is>
       </c>
       <c r="B153" s="3" t="inlineStr">
@@ -9868,7 +9874,7 @@
         </is>
       </c>
       <c r="D153" s="4" t="n">
-        <v>12.65</v>
+        <v>4.6</v>
       </c>
       <c r="E153" s="5" t="n">
         <v>1.0016</v>
@@ -10319,12 +10325,12 @@
     <row r="160">
       <c r="A160" s="3" t="inlineStr">
         <is>
-          <t>EASTCRK</t>
+          <t>EASTCRK2</t>
         </is>
       </c>
       <c r="B160" s="3" t="inlineStr">
         <is>
-          <t>Eastern Creek LFG PS Units 1-4</t>
+          <t>Eastern Creek 2 Gas Utilisation Facility</t>
         </is>
       </c>
       <c r="C160" s="3" t="inlineStr">
@@ -10333,22 +10339,22 @@
         </is>
       </c>
       <c r="D160" s="4" t="n">
-        <v>5.056</v>
+        <v>6.738</v>
       </c>
       <c r="E160" s="5" t="n">
-        <v>1.0018</v>
+        <v>1.0021</v>
       </c>
       <c r="F160" s="5" t="n">
-        <v>1.0035</v>
+        <v>1.0021</v>
       </c>
       <c r="G160" s="5" t="n">
-        <v>1.0041</v>
+        <v>1.0021</v>
       </c>
       <c r="H160" s="5" t="n">
-        <v>1.0033</v>
+        <v>1.0021</v>
       </c>
       <c r="I160" s="5" t="n">
-        <v>1.001</v>
+        <v>1.0021</v>
       </c>
       <c r="J160" s="5" t="n">
         <v>1.001</v>
@@ -10386,12 +10392,12 @@
     <row r="161">
       <c r="A161" s="3" t="inlineStr">
         <is>
-          <t>EASTCRK2</t>
+          <t>EASTCRK</t>
         </is>
       </c>
       <c r="B161" s="3" t="inlineStr">
         <is>
-          <t>Eastern Creek 2 Gas Utilisation Facility</t>
+          <t>Eastern Creek LFG PS Units 1-4</t>
         </is>
       </c>
       <c r="C161" s="3" t="inlineStr">
@@ -10400,22 +10406,22 @@
         </is>
       </c>
       <c r="D161" s="4" t="n">
-        <v>6.738</v>
+        <v>5.056</v>
       </c>
       <c r="E161" s="5" t="n">
-        <v>1.0021</v>
+        <v>1.0018</v>
       </c>
       <c r="F161" s="5" t="n">
-        <v>1.0021</v>
+        <v>1.0035</v>
       </c>
       <c r="G161" s="5" t="n">
-        <v>1.0021</v>
+        <v>1.0041</v>
       </c>
       <c r="H161" s="5" t="n">
-        <v>1.0021</v>
+        <v>1.0033</v>
       </c>
       <c r="I161" s="5" t="n">
-        <v>1.0021</v>
+        <v>1.001</v>
       </c>
       <c r="J161" s="5" t="n">
         <v>1.001</v>
@@ -10634,21 +10640,21 @@
     <row r="165">
       <c r="A165" s="3" t="inlineStr">
         <is>
-          <t>TARALGA1</t>
+          <t>WDLNGN01</t>
         </is>
       </c>
       <c r="B165" s="3" t="inlineStr">
         <is>
-          <t>Taralga Wind Farm</t>
+          <t>Woodlawn Bioreactor Energy Generation Station</t>
         </is>
       </c>
       <c r="C165" s="3" t="inlineStr">
         <is>
-          <t>Wind</t>
+          <t>Other Renewable</t>
         </is>
       </c>
       <c r="D165" s="4" t="n">
-        <v>106.8</v>
+        <v>7</v>
       </c>
       <c r="E165" s="5" t="n">
         <v>0.9844000000000001</v>
@@ -10701,21 +10707,21 @@
     <row r="166">
       <c r="A166" s="3" t="inlineStr">
         <is>
-          <t>WDLNGN01</t>
+          <t>TARALGA1</t>
         </is>
       </c>
       <c r="B166" s="3" t="inlineStr">
         <is>
-          <t>Woodlawn Bioreactor Energy Generation Station</t>
+          <t>Taralga Wind Farm</t>
         </is>
       </c>
       <c r="C166" s="3" t="inlineStr">
         <is>
-          <t>Other Renewable</t>
+          <t>Wind</t>
         </is>
       </c>
       <c r="D166" s="4" t="n">
-        <v>7</v>
+        <v>106.8</v>
       </c>
       <c r="E166" s="5" t="n">
         <v>0.9844000000000001</v>
@@ -10886,7 +10892,7 @@
     <row r="169">
       <c r="A169" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-4</t>
+          <t>TUMUT3-6</t>
         </is>
       </c>
       <c r="B169" s="3" t="inlineStr">
@@ -10949,7 +10955,7 @@
     <row r="170">
       <c r="A170" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-3</t>
+          <t>TUMUT3-5</t>
         </is>
       </c>
       <c r="B170" s="3" t="inlineStr">
@@ -11012,7 +11018,7 @@
     <row r="171">
       <c r="A171" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-5</t>
+          <t>TUMUT3-4</t>
         </is>
       </c>
       <c r="B171" s="3" t="inlineStr">
@@ -11075,7 +11081,7 @@
     <row r="172">
       <c r="A172" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-1</t>
+          <t>TUMUT3-2</t>
         </is>
       </c>
       <c r="B172" s="3" t="inlineStr">
@@ -11138,7 +11144,7 @@
     <row r="173">
       <c r="A173" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-2</t>
+          <t>TUMUT3-3</t>
         </is>
       </c>
       <c r="B173" s="3" t="inlineStr">
@@ -11201,7 +11207,7 @@
     <row r="174">
       <c r="A174" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-6</t>
+          <t>TUMUT3-1</t>
         </is>
       </c>
       <c r="B174" s="3" t="inlineStr">
@@ -11487,42 +11493,38 @@
     <row r="180">
       <c r="A180" s="3" t="inlineStr">
         <is>
-          <t>TERALBA</t>
+          <t>HVGTS</t>
         </is>
       </c>
       <c r="B180" s="3" t="inlineStr">
         <is>
-          <t>TERALBA POWER STATION</t>
-        </is>
-      </c>
-      <c r="C180" s="3" t="inlineStr">
-        <is>
-          <t>Other Renewable</t>
-        </is>
-      </c>
-      <c r="D180" s="4" t="n">
-        <v>3</v>
-      </c>
+          <t>Hunter Valley Gas Turbine</t>
+        </is>
+      </c>
+      <c r="C180" s="3" t="n">
+        <v/>
+      </c>
+      <c r="D180" s="3" t="inlineStr"/>
       <c r="E180" s="5" t="n">
-        <v>0.9926</v>
+        <v>0.974</v>
       </c>
       <c r="F180" s="5" t="n">
-        <v>0.9907</v>
+        <v>0.9679</v>
       </c>
       <c r="G180" s="5" t="n">
-        <v>0.9892</v>
+        <v>0.9582000000000001</v>
       </c>
       <c r="H180" s="5" t="n">
-        <v>0.9901</v>
+        <v>0.9596</v>
       </c>
       <c r="I180" s="5" t="n">
-        <v>0.9903999999999999</v>
+        <v>0.9654</v>
       </c>
       <c r="J180" s="5" t="n">
-        <v>0.9907</v>
+        <v>0.9673</v>
       </c>
       <c r="K180" s="5" t="n">
-        <v>0.9917</v>
+        <v>0.9651999999999999</v>
       </c>
       <c r="L180" s="5" t="inlineStr"/>
       <c r="M180" s="5" t="inlineStr"/>
@@ -11540,12 +11542,12 @@
     <row r="181">
       <c r="A181" s="3" t="inlineStr">
         <is>
-          <t>WOYWOY1</t>
+          <t>KINCUM1</t>
         </is>
       </c>
       <c r="B181" s="3" t="inlineStr">
         <is>
-          <t>Woy Woy Landfill Site</t>
+          <t>Kincumber Landfill Site</t>
         </is>
       </c>
       <c r="C181" s="3" t="inlineStr">
@@ -11593,38 +11595,42 @@
     <row r="182">
       <c r="A182" s="3" t="inlineStr">
         <is>
-          <t>HVGTS</t>
+          <t>AGLNOW1</t>
         </is>
       </c>
       <c r="B182" s="3" t="inlineStr">
         <is>
-          <t>Hunter Valley Gas Turbine</t>
-        </is>
-      </c>
-      <c r="C182" s="3" t="n">
-        <v/>
-      </c>
-      <c r="D182" s="3" t="inlineStr"/>
+          <t>West Nowra Landfill Gas Power Generation Facility</t>
+        </is>
+      </c>
+      <c r="C182" s="3" t="inlineStr">
+        <is>
+          <t>Other Renewable</t>
+        </is>
+      </c>
+      <c r="D182" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="E182" s="5" t="n">
-        <v>0.974</v>
+        <v>0.9916</v>
       </c>
       <c r="F182" s="5" t="n">
-        <v>0.9679</v>
+        <v>0.9986</v>
       </c>
       <c r="G182" s="5" t="n">
-        <v>0.9582000000000001</v>
+        <v>1.0023</v>
       </c>
       <c r="H182" s="5" t="n">
-        <v>0.9596</v>
+        <v>1.0037</v>
       </c>
       <c r="I182" s="5" t="n">
-        <v>0.9654</v>
+        <v>0.9929</v>
       </c>
       <c r="J182" s="5" t="n">
-        <v>0.9673</v>
+        <v>0.9967</v>
       </c>
       <c r="K182" s="5" t="n">
-        <v>0.9651999999999999</v>
+        <v>0.9929</v>
       </c>
       <c r="L182" s="5" t="inlineStr"/>
       <c r="M182" s="5" t="inlineStr"/>
@@ -11693,42 +11699,42 @@
     <row r="184">
       <c r="A184" s="3" t="inlineStr">
         <is>
-          <t>AGLNOW1</t>
+          <t>LD03</t>
         </is>
       </c>
       <c r="B184" s="3" t="inlineStr">
         <is>
-          <t>West Nowra Landfill Gas Power Generation Facility</t>
+          <t>Liddell Power Station</t>
         </is>
       </c>
       <c r="C184" s="3" t="inlineStr">
         <is>
-          <t>Other Renewable</t>
+          <t>Fossil</t>
         </is>
       </c>
       <c r="D184" s="4" t="n">
-        <v>1</v>
+        <v>500</v>
       </c>
       <c r="E184" s="5" t="n">
-        <v>0.9916</v>
+        <v>0.9676</v>
       </c>
       <c r="F184" s="5" t="n">
-        <v>0.9986</v>
+        <v>0.9593</v>
       </c>
       <c r="G184" s="5" t="n">
-        <v>1.0023</v>
+        <v>0.9509</v>
       </c>
       <c r="H184" s="5" t="n">
-        <v>1.0037</v>
+        <v>0.9537</v>
       </c>
       <c r="I184" s="5" t="n">
-        <v>0.9929</v>
+        <v>0.9593</v>
       </c>
       <c r="J184" s="5" t="n">
-        <v>0.9967</v>
+        <v>0.9631</v>
       </c>
       <c r="K184" s="5" t="n">
-        <v>0.9929</v>
+        <v>0.9628</v>
       </c>
       <c r="L184" s="5" t="inlineStr"/>
       <c r="M184" s="5" t="inlineStr"/>
@@ -11746,12 +11752,12 @@
     <row r="185">
       <c r="A185" s="3" t="inlineStr">
         <is>
-          <t>KINCUM1</t>
+          <t>TERALBA</t>
         </is>
       </c>
       <c r="B185" s="3" t="inlineStr">
         <is>
-          <t>Kincumber Landfill Site</t>
+          <t>TERALBA POWER STATION</t>
         </is>
       </c>
       <c r="C185" s="3" t="inlineStr">
@@ -11760,28 +11766,28 @@
         </is>
       </c>
       <c r="D185" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E185" s="5" t="n">
-        <v>1.0017</v>
+        <v>0.9926</v>
       </c>
       <c r="F185" s="5" t="n">
-        <v>1.0015</v>
+        <v>0.9907</v>
       </c>
       <c r="G185" s="5" t="n">
-        <v>1.0008</v>
+        <v>0.9892</v>
       </c>
       <c r="H185" s="5" t="n">
-        <v>1.0011</v>
+        <v>0.9901</v>
       </c>
       <c r="I185" s="5" t="n">
-        <v>1.0036</v>
+        <v>0.9903999999999999</v>
       </c>
       <c r="J185" s="5" t="n">
-        <v>1.0019</v>
+        <v>0.9907</v>
       </c>
       <c r="K185" s="5" t="n">
-        <v>1.0037</v>
+        <v>0.9917</v>
       </c>
       <c r="L185" s="5" t="inlineStr"/>
       <c r="M185" s="5" t="inlineStr"/>
@@ -11799,42 +11805,42 @@
     <row r="186">
       <c r="A186" s="3" t="inlineStr">
         <is>
-          <t>LD03</t>
+          <t>WOYWOY1</t>
         </is>
       </c>
       <c r="B186" s="3" t="inlineStr">
         <is>
-          <t>Liddell Power Station</t>
+          <t>Woy Woy Landfill Site</t>
         </is>
       </c>
       <c r="C186" s="3" t="inlineStr">
         <is>
-          <t>Fossil</t>
+          <t>Other Renewable</t>
         </is>
       </c>
       <c r="D186" s="4" t="n">
-        <v>500</v>
+        <v>1</v>
       </c>
       <c r="E186" s="5" t="n">
-        <v>0.9676</v>
+        <v>1.0017</v>
       </c>
       <c r="F186" s="5" t="n">
-        <v>0.9593</v>
+        <v>1.0015</v>
       </c>
       <c r="G186" s="5" t="n">
-        <v>0.9509</v>
+        <v>1.0008</v>
       </c>
       <c r="H186" s="5" t="n">
-        <v>0.9537</v>
+        <v>1.0011</v>
       </c>
       <c r="I186" s="5" t="n">
-        <v>0.9593</v>
+        <v>1.0036</v>
       </c>
       <c r="J186" s="5" t="n">
-        <v>0.9631</v>
+        <v>1.0019</v>
       </c>
       <c r="K186" s="5" t="n">
-        <v>0.9628</v>
+        <v>1.0037</v>
       </c>
       <c r="L186" s="5" t="inlineStr"/>
       <c r="M186" s="5" t="inlineStr"/>
@@ -11907,7 +11913,7 @@
     <row r="188">
       <c r="A188" s="3" t="inlineStr">
         <is>
-          <t>LD02</t>
+          <t>LD01</t>
         </is>
       </c>
       <c r="B188" s="3" t="inlineStr">
@@ -11962,7 +11968,7 @@
     <row r="189">
       <c r="A189" s="3" t="inlineStr">
         <is>
-          <t>LD01</t>
+          <t>LD02</t>
         </is>
       </c>
       <c r="B189" s="3" t="inlineStr">
@@ -12017,21 +12023,21 @@
     <row r="190">
       <c r="A190" s="3" t="inlineStr">
         <is>
-          <t>WALGRVG1</t>
+          <t>MLLFGEF1</t>
         </is>
       </c>
       <c r="B190" s="3" t="inlineStr">
         <is>
-          <t>Wallgrove BESS 1</t>
+          <t>Mugga Lane Landfill Gas To Energy Facility</t>
         </is>
       </c>
       <c r="C190" s="3" t="inlineStr">
         <is>
-          <t>Battery</t>
+          <t>Other Renewable</t>
         </is>
       </c>
       <c r="D190" s="4" t="n">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="E190" s="5" t="inlineStr"/>
       <c r="F190" s="5" t="inlineStr"/>
@@ -12040,16 +12046,16 @@
       <c r="I190" s="5" t="inlineStr"/>
       <c r="J190" s="5" t="inlineStr"/>
       <c r="K190" s="5" t="n">
-        <v>1.0011</v>
+        <v>0.9683</v>
       </c>
       <c r="L190" s="5" t="n">
-        <v>1.001</v>
+        <v>0.9687</v>
       </c>
       <c r="M190" s="5" t="n">
-        <v>1.001</v>
+        <v>0.9663</v>
       </c>
       <c r="N190" s="5" t="n">
-        <v>1.001</v>
+        <v>0.9567</v>
       </c>
       <c r="O190" s="5" t="inlineStr"/>
       <c r="P190" s="5" t="inlineStr"/>
@@ -12064,21 +12070,21 @@
     <row r="191">
       <c r="A191" s="3" t="inlineStr">
         <is>
-          <t>MLLFGEF1</t>
+          <t>DPNTBG1</t>
         </is>
       </c>
       <c r="B191" s="3" t="inlineStr">
         <is>
-          <t>Mugga Lane Landfill Gas To Energy Facility</t>
+          <t>Darlington Point Energy Storage System</t>
         </is>
       </c>
       <c r="C191" s="3" t="inlineStr">
         <is>
-          <t>Other Renewable</t>
+          <t>Battery</t>
         </is>
       </c>
       <c r="D191" s="4" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="E191" s="5" t="inlineStr"/>
       <c r="F191" s="5" t="inlineStr"/>
@@ -12086,17 +12092,15 @@
       <c r="H191" s="5" t="inlineStr"/>
       <c r="I191" s="5" t="inlineStr"/>
       <c r="J191" s="5" t="inlineStr"/>
-      <c r="K191" s="5" t="n">
-        <v>0.9683</v>
-      </c>
+      <c r="K191" s="5" t="inlineStr"/>
       <c r="L191" s="5" t="n">
-        <v>0.9687</v>
+        <v>0.9402</v>
       </c>
       <c r="M191" s="5" t="n">
-        <v>0.9663</v>
+        <v>0.9089</v>
       </c>
       <c r="N191" s="5" t="n">
-        <v>0.9567</v>
+        <v>0.9048</v>
       </c>
       <c r="O191" s="5" t="inlineStr"/>
       <c r="P191" s="5" t="inlineStr"/>
@@ -12111,12 +12115,12 @@
     <row r="192">
       <c r="A192" s="3" t="inlineStr">
         <is>
-          <t>BHBG1</t>
+          <t>RESS1G</t>
         </is>
       </c>
       <c r="B192" s="3" t="inlineStr">
         <is>
-          <t>Broken Hill Battery Energy Storage System</t>
+          <t>Riverina BESS 1</t>
         </is>
       </c>
       <c r="C192" s="3" t="inlineStr">
@@ -12125,7 +12129,7 @@
         </is>
       </c>
       <c r="D192" s="4" t="n">
-        <v>66</v>
+        <v>80</v>
       </c>
       <c r="E192" s="5" t="inlineStr"/>
       <c r="F192" s="5" t="inlineStr"/>
@@ -12134,12 +12138,14 @@
       <c r="I192" s="5" t="inlineStr"/>
       <c r="J192" s="5" t="inlineStr"/>
       <c r="K192" s="5" t="inlineStr"/>
-      <c r="L192" s="5" t="inlineStr"/>
+      <c r="L192" s="5" t="n">
+        <v>0.9286</v>
+      </c>
       <c r="M192" s="5" t="n">
-        <v>0.8671</v>
+        <v>0.9089</v>
       </c>
       <c r="N192" s="5" t="n">
-        <v>0.8423</v>
+        <v>0.8702</v>
       </c>
       <c r="O192" s="5" t="inlineStr"/>
       <c r="P192" s="5" t="inlineStr"/>
@@ -12154,12 +12160,12 @@
     <row r="193">
       <c r="A193" s="3" t="inlineStr">
         <is>
-          <t>CAPBES1G</t>
+          <t>RIVNBG2</t>
         </is>
       </c>
       <c r="B193" s="3" t="inlineStr">
         <is>
-          <t>Capital Battery</t>
+          <t>Riverina Energy Storage System 2</t>
         </is>
       </c>
       <c r="C193" s="3" t="inlineStr">
@@ -12168,7 +12174,7 @@
         </is>
       </c>
       <c r="D193" s="4" t="n">
-        <v>125</v>
+        <v>65</v>
       </c>
       <c r="E193" s="5" t="inlineStr"/>
       <c r="F193" s="5" t="inlineStr"/>
@@ -12177,12 +12183,14 @@
       <c r="I193" s="5" t="inlineStr"/>
       <c r="J193" s="5" t="inlineStr"/>
       <c r="K193" s="5" t="inlineStr"/>
-      <c r="L193" s="5" t="inlineStr"/>
+      <c r="L193" s="5" t="n">
+        <v>0.9058</v>
+      </c>
       <c r="M193" s="5" t="n">
-        <v>0.9704</v>
+        <v>0.9106</v>
       </c>
       <c r="N193" s="5" t="n">
-        <v>0.9337</v>
+        <v>0.9048</v>
       </c>
       <c r="O193" s="5" t="inlineStr"/>
       <c r="P193" s="5" t="inlineStr"/>
@@ -12197,12 +12205,12 @@
     <row r="194">
       <c r="A194" s="3" t="inlineStr">
         <is>
-          <t>QBYNBG1</t>
+          <t>WALGRVG1</t>
         </is>
       </c>
       <c r="B194" s="3" t="inlineStr">
         <is>
-          <t>Queanbeyan BESS</t>
+          <t>Wallgrove BESS 1</t>
         </is>
       </c>
       <c r="C194" s="3" t="inlineStr">
@@ -12211,7 +12219,7 @@
         </is>
       </c>
       <c r="D194" s="4" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="E194" s="5" t="inlineStr"/>
       <c r="F194" s="5" t="inlineStr"/>
@@ -12219,15 +12227,17 @@
       <c r="H194" s="5" t="inlineStr"/>
       <c r="I194" s="5" t="inlineStr"/>
       <c r="J194" s="5" t="inlineStr"/>
-      <c r="K194" s="5" t="inlineStr"/>
+      <c r="K194" s="5" t="n">
+        <v>1.0011</v>
+      </c>
       <c r="L194" s="5" t="n">
-        <v>0.9752</v>
+        <v>1.001</v>
       </c>
       <c r="M194" s="5" t="n">
-        <v>0.979</v>
+        <v>1.001</v>
       </c>
       <c r="N194" s="5" t="n">
-        <v>0.9571</v>
+        <v>1.001</v>
       </c>
       <c r="O194" s="5" t="inlineStr"/>
       <c r="P194" s="5" t="inlineStr"/>
@@ -12242,12 +12252,12 @@
     <row r="195">
       <c r="A195" s="3" t="inlineStr">
         <is>
-          <t>RIVNBG2</t>
+          <t>BHBG1</t>
         </is>
       </c>
       <c r="B195" s="3" t="inlineStr">
         <is>
-          <t>Riverina Energy Storage System 2</t>
+          <t>Broken Hill Battery Energy Storage System</t>
         </is>
       </c>
       <c r="C195" s="3" t="inlineStr">
@@ -12256,7 +12266,7 @@
         </is>
       </c>
       <c r="D195" s="4" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E195" s="5" t="inlineStr"/>
       <c r="F195" s="5" t="inlineStr"/>
@@ -12265,14 +12275,12 @@
       <c r="I195" s="5" t="inlineStr"/>
       <c r="J195" s="5" t="inlineStr"/>
       <c r="K195" s="5" t="inlineStr"/>
-      <c r="L195" s="5" t="n">
-        <v>0.9058</v>
-      </c>
+      <c r="L195" s="5" t="inlineStr"/>
       <c r="M195" s="5" t="n">
-        <v>0.9106</v>
+        <v>0.8671</v>
       </c>
       <c r="N195" s="5" t="n">
-        <v>0.9048</v>
+        <v>0.8423</v>
       </c>
       <c r="O195" s="5" t="inlineStr"/>
       <c r="P195" s="5" t="inlineStr"/>
@@ -12287,12 +12295,12 @@
     <row r="196">
       <c r="A196" s="3" t="inlineStr">
         <is>
-          <t>DPNTBG1</t>
+          <t>QBYNBG1</t>
         </is>
       </c>
       <c r="B196" s="3" t="inlineStr">
         <is>
-          <t>Darlington Point Energy Storage System</t>
+          <t>Queanbeyan BESS</t>
         </is>
       </c>
       <c r="C196" s="3" t="inlineStr">
@@ -12301,7 +12309,7 @@
         </is>
       </c>
       <c r="D196" s="4" t="n">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="E196" s="5" t="inlineStr"/>
       <c r="F196" s="5" t="inlineStr"/>
@@ -12311,13 +12319,13 @@
       <c r="J196" s="5" t="inlineStr"/>
       <c r="K196" s="5" t="inlineStr"/>
       <c r="L196" s="5" t="n">
-        <v>0.9402</v>
+        <v>0.9752</v>
       </c>
       <c r="M196" s="5" t="n">
-        <v>0.9089</v>
+        <v>0.979</v>
       </c>
       <c r="N196" s="5" t="n">
-        <v>0.9048</v>
+        <v>0.9571</v>
       </c>
       <c r="O196" s="5" t="inlineStr"/>
       <c r="P196" s="5" t="inlineStr"/>
@@ -12332,12 +12340,12 @@
     <row r="197">
       <c r="A197" s="3" t="inlineStr">
         <is>
-          <t>RESS1G</t>
+          <t>CAPBES1G</t>
         </is>
       </c>
       <c r="B197" s="3" t="inlineStr">
         <is>
-          <t>Riverina BESS 1</t>
+          <t>Capital Battery</t>
         </is>
       </c>
       <c r="C197" s="3" t="inlineStr">
@@ -12346,7 +12354,7 @@
         </is>
       </c>
       <c r="D197" s="4" t="n">
-        <v>80</v>
+        <v>125</v>
       </c>
       <c r="E197" s="5" t="inlineStr"/>
       <c r="F197" s="5" t="inlineStr"/>
@@ -12355,14 +12363,12 @@
       <c r="I197" s="5" t="inlineStr"/>
       <c r="J197" s="5" t="inlineStr"/>
       <c r="K197" s="5" t="inlineStr"/>
-      <c r="L197" s="5" t="n">
-        <v>0.9286</v>
-      </c>
+      <c r="L197" s="5" t="inlineStr"/>
       <c r="M197" s="5" t="n">
-        <v>0.9089</v>
+        <v>0.9704</v>
       </c>
       <c r="N197" s="5" t="n">
-        <v>0.8702</v>
+        <v>0.9337</v>
       </c>
       <c r="O197" s="5" t="inlineStr"/>
       <c r="P197" s="5" t="inlineStr"/>
@@ -12626,14 +12632,12 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>WRWF1</t>
+          <t>WRSF1</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr"/>
       <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="n">
-        <v>0.8468</v>
-      </c>
+      <c r="D4" s="5" t="inlineStr"/>
       <c r="E4" s="5" t="n">
         <v>0.8427</v>
       </c>
@@ -12668,12 +12672,14 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>WRSF1</t>
+          <t>WRWF1</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr"/>
       <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="n">
+        <v>0.8468</v>
+      </c>
       <c r="E5" s="5" t="n">
         <v>0.8427</v>
       </c>
@@ -13362,7 +13368,7 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>WYASF1</t>
+          <t>WSTWYSF1</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr"/>
@@ -13394,7 +13400,7 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>WSTWYSF1</t>
+          <t>WYASF1</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr"/>
@@ -13546,7 +13552,7 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>NEWENSF2</t>
+          <t>NEWENSF1</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr"/>
@@ -13578,7 +13584,7 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>NEWENSF1</t>
+          <t>NEWENSF2</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr"/>
@@ -13610,15 +13616,19 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>GOONSF1</t>
+          <t>PARSF1</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr"/>
       <c r="C31" s="5" t="inlineStr"/>
-      <c r="D31" s="5" t="inlineStr"/>
-      <c r="E31" s="5" t="inlineStr"/>
+      <c r="D31" s="5" t="n">
+        <v>1.0135</v>
+      </c>
+      <c r="E31" s="5" t="n">
+        <v>0.9964</v>
+      </c>
       <c r="F31" s="5" t="n">
-        <v>0.9791</v>
+        <v>0.9812</v>
       </c>
       <c r="G31" s="5" t="n">
         <v>0.9258999999999999</v>
@@ -13648,19 +13658,15 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>PARSF1</t>
+          <t>GOONSF1</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr"/>
       <c r="C32" s="5" t="inlineStr"/>
-      <c r="D32" s="5" t="n">
-        <v>1.0135</v>
-      </c>
-      <c r="E32" s="5" t="n">
-        <v>0.9964</v>
-      </c>
+      <c r="D32" s="5" t="inlineStr"/>
+      <c r="E32" s="5" t="inlineStr"/>
       <c r="F32" s="5" t="n">
-        <v>0.9812</v>
+        <v>0.9791</v>
       </c>
       <c r="G32" s="5" t="n">
         <v>0.9258999999999999</v>
@@ -13840,7 +13846,7 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>QPSFB2</t>
+          <t>QPSFB1</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr"/>
@@ -13863,14 +13869,12 @@
       <c r="O37" s="5" t="n">
         <v>0.9032</v>
       </c>
-      <c r="P37" s="5" t="n">
-        <v>0.9032</v>
-      </c>
+      <c r="P37" s="5" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>QPSFB1</t>
+          <t>QPSFB2</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr"/>
@@ -13893,7 +13897,9 @@
       <c r="O38" s="5" t="n">
         <v>0.9032</v>
       </c>
-      <c r="P38" s="5" t="inlineStr"/>
+      <c r="P38" s="5" t="n">
+        <v>0.9032</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -14038,7 +14044,7 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>URANQ13</t>
+          <t>URANQ14</t>
         </is>
       </c>
       <c r="B43" s="5" t="n">
@@ -14176,7 +14182,7 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>URANQ14</t>
+          <t>URANQ13</t>
         </is>
       </c>
       <c r="B46" s="5" t="n">
@@ -14298,38 +14304,42 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>SKSF1</t>
-        </is>
-      </c>
-      <c r="B49" s="5" t="inlineStr"/>
-      <c r="C49" s="5" t="inlineStr"/>
+          <t>GUTHEGA</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0.8882</v>
+      </c>
+      <c r="C49" s="5" t="n">
+        <v>0.9371</v>
+      </c>
       <c r="D49" s="5" t="n">
-        <v>0.9714</v>
+        <v>0.9658</v>
       </c>
       <c r="E49" s="5" t="n">
-        <v>0.9708</v>
+        <v>0.9537</v>
       </c>
       <c r="F49" s="5" t="n">
-        <v>0.9603</v>
+        <v>0.9016</v>
       </c>
       <c r="G49" s="5" t="n">
-        <v>0.9569</v>
+        <v>0.9125</v>
       </c>
       <c r="H49" s="5" t="n">
-        <v>0.9444</v>
+        <v>0.9006</v>
       </c>
       <c r="I49" s="5" t="n">
-        <v>0.9352</v>
+        <v>0.887</v>
       </c>
       <c r="J49" s="5" t="n">
-        <v>0.9439</v>
+        <v>0.893</v>
       </c>
       <c r="K49" s="5" t="n">
-        <v>0.9284</v>
+        <v>0.892</v>
       </c>
       <c r="L49" s="5" t="inlineStr"/>
       <c r="M49" s="5" t="n">
-        <v>0.923</v>
+        <v>0.9135</v>
       </c>
       <c r="N49" s="5" t="inlineStr"/>
       <c r="O49" s="5" t="n">
@@ -14340,15 +14350,19 @@
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>NEVERSF1</t>
+          <t>SKSF1</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr"/>
       <c r="C50" s="5" t="inlineStr"/>
-      <c r="D50" s="5" t="inlineStr"/>
-      <c r="E50" s="5" t="inlineStr"/>
+      <c r="D50" s="5" t="n">
+        <v>0.9714</v>
+      </c>
+      <c r="E50" s="5" t="n">
+        <v>0.9708</v>
+      </c>
       <c r="F50" s="5" t="n">
-        <v>0.9582000000000001</v>
+        <v>0.9603</v>
       </c>
       <c r="G50" s="5" t="n">
         <v>0.9569</v>
@@ -14378,22 +14392,16 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>NASF1</t>
+          <t>WELLSF1</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr"/>
       <c r="C51" s="5" t="inlineStr"/>
-      <c r="D51" s="5" t="n">
-        <v>0.9714</v>
-      </c>
-      <c r="E51" s="5" t="n">
-        <v>0.9708</v>
-      </c>
-      <c r="F51" s="5" t="n">
-        <v>0.9603</v>
-      </c>
+      <c r="D51" s="5" t="inlineStr"/>
+      <c r="E51" s="5" t="inlineStr"/>
+      <c r="F51" s="5" t="inlineStr"/>
       <c r="G51" s="5" t="n">
-        <v>0.9569</v>
+        <v>0.9471000000000001</v>
       </c>
       <c r="H51" s="5" t="n">
         <v>0.9444</v>
@@ -14420,16 +14428,18 @@
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>WELLSF1</t>
+          <t>NEVERSF1</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr"/>
       <c r="C52" s="5" t="inlineStr"/>
       <c r="D52" s="5" t="inlineStr"/>
       <c r="E52" s="5" t="inlineStr"/>
-      <c r="F52" s="5" t="inlineStr"/>
+      <c r="F52" s="5" t="n">
+        <v>0.9582000000000001</v>
+      </c>
       <c r="G52" s="5" t="n">
-        <v>0.9471000000000001</v>
+        <v>0.9569</v>
       </c>
       <c r="H52" s="5" t="n">
         <v>0.9444</v>
@@ -14456,42 +14466,38 @@
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>GUTHEGA</t>
-        </is>
-      </c>
-      <c r="B53" s="5" t="n">
-        <v>0.8882</v>
-      </c>
-      <c r="C53" s="5" t="n">
-        <v>0.9371</v>
-      </c>
+          <t>NASF1</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr"/>
+      <c r="C53" s="5" t="inlineStr"/>
       <c r="D53" s="5" t="n">
-        <v>0.9658</v>
+        <v>0.9714</v>
       </c>
       <c r="E53" s="5" t="n">
-        <v>0.9537</v>
+        <v>0.9708</v>
       </c>
       <c r="F53" s="5" t="n">
-        <v>0.9016</v>
+        <v>0.9603</v>
       </c>
       <c r="G53" s="5" t="n">
-        <v>0.9125</v>
+        <v>0.9569</v>
       </c>
       <c r="H53" s="5" t="n">
-        <v>0.9006</v>
+        <v>0.9444</v>
       </c>
       <c r="I53" s="5" t="n">
-        <v>0.887</v>
+        <v>0.9352</v>
       </c>
       <c r="J53" s="5" t="n">
-        <v>0.893</v>
+        <v>0.9439</v>
       </c>
       <c r="K53" s="5" t="n">
-        <v>0.892</v>
+        <v>0.9284</v>
       </c>
       <c r="L53" s="5" t="inlineStr"/>
       <c r="M53" s="5" t="n">
-        <v>0.9135</v>
+        <v>0.923</v>
       </c>
       <c r="N53" s="5" t="inlineStr"/>
       <c r="O53" s="5" t="n">
@@ -15008,7 +15014,7 @@
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>CULLRGWF</t>
+          <t>GUNNING1</t>
         </is>
       </c>
       <c r="B67" s="5" t="n">
@@ -15054,7 +15060,7 @@
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>GUNNING1</t>
+          <t>CULLRGWF</t>
         </is>
       </c>
       <c r="B68" s="5" t="n">
@@ -15124,7 +15130,7 @@
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>HUNTER2</t>
+          <t>HUNTER1</t>
         </is>
       </c>
       <c r="B70" s="5" t="inlineStr"/>
@@ -15152,7 +15158,7 @@
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>HUNTER1</t>
+          <t>HUNTER2</t>
         </is>
       </c>
       <c r="B71" s="5" t="inlineStr"/>
@@ -16066,7 +16072,7 @@
     <row r="94">
       <c r="A94" s="3" t="inlineStr">
         <is>
-          <t>WOODLWN1</t>
+          <t>CAPTL_WF</t>
         </is>
       </c>
       <c r="B94" s="5" t="n">
@@ -16112,7 +16118,7 @@
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>CAPTL_WF</t>
+          <t>WOODLWN1</t>
         </is>
       </c>
       <c r="B95" s="5" t="n">
@@ -16204,7 +16210,7 @@
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t>NYNGAN1</t>
+          <t>BDONGHYD</t>
         </is>
       </c>
       <c r="B97" s="5" t="n">
@@ -16250,7 +16256,7 @@
     <row r="98">
       <c r="A98" s="3" t="inlineStr">
         <is>
-          <t>BDONGHYD</t>
+          <t>NYNGAN1</t>
         </is>
       </c>
       <c r="B98" s="5" t="n">
@@ -16386,7 +16392,7 @@
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>MP2</t>
+          <t>MP1</t>
         </is>
       </c>
       <c r="B101" s="5" t="n">
@@ -16432,7 +16438,7 @@
     <row r="102">
       <c r="A102" s="3" t="inlineStr">
         <is>
-          <t>MP1</t>
+          <t>MP2</t>
         </is>
       </c>
       <c r="B102" s="5" t="n">
@@ -16478,7 +16484,7 @@
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>GLBWNHYD</t>
+          <t>GLENNCRK</t>
         </is>
       </c>
       <c r="B103" s="5" t="n">
@@ -16524,7 +16530,7 @@
     <row r="104">
       <c r="A104" s="3" t="inlineStr">
         <is>
-          <t>GLENNCRK</t>
+          <t>GLBWNHYD</t>
         </is>
       </c>
       <c r="B104" s="5" t="n">
@@ -16604,7 +16610,7 @@
     <row r="106">
       <c r="A106" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1-1</t>
+          <t>TUMUT2-4</t>
         </is>
       </c>
       <c r="B106" s="5" t="n">
@@ -16650,7 +16656,7 @@
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1-2</t>
+          <t>TUMUT2-1</t>
         </is>
       </c>
       <c r="B107" s="5" t="n">
@@ -16696,7 +16702,7 @@
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1-3</t>
+          <t>TUMUT1-4</t>
         </is>
       </c>
       <c r="B108" s="5" t="n">
@@ -16742,7 +16748,7 @@
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2-4</t>
+          <t>TUMUT2-3</t>
         </is>
       </c>
       <c r="B109" s="5" t="n">
@@ -16834,7 +16840,7 @@
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2-1</t>
+          <t>TUMUT1-3</t>
         </is>
       </c>
       <c r="B111" s="5" t="n">
@@ -16880,7 +16886,7 @@
     <row r="112">
       <c r="A112" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1-4</t>
+          <t>TUMUT1-1</t>
         </is>
       </c>
       <c r="B112" s="5" t="n">
@@ -16926,7 +16932,7 @@
     <row r="113">
       <c r="A113" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2-3</t>
+          <t>TUMUT1-2</t>
         </is>
       </c>
       <c r="B113" s="5" t="n">
@@ -17074,7 +17080,7 @@
     <row r="117">
       <c r="A117" s="3" t="inlineStr">
         <is>
-          <t>CG3</t>
+          <t>CG1</t>
         </is>
       </c>
       <c r="B117" s="5" t="n">
@@ -17120,7 +17126,7 @@
     <row r="118">
       <c r="A118" s="3" t="inlineStr">
         <is>
-          <t>CG2</t>
+          <t>CG3</t>
         </is>
       </c>
       <c r="B118" s="5" t="n">
@@ -17166,7 +17172,7 @@
     <row r="119">
       <c r="A119" s="3" t="inlineStr">
         <is>
-          <t>CG4</t>
+          <t>CG2</t>
         </is>
       </c>
       <c r="B119" s="5" t="n">
@@ -17212,7 +17218,7 @@
     <row r="120">
       <c r="A120" s="3" t="inlineStr">
         <is>
-          <t>CG1</t>
+          <t>CG4</t>
         </is>
       </c>
       <c r="B120" s="5" t="n">
@@ -17292,7 +17298,7 @@
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
         <is>
-          <t>ERGT01</t>
+          <t>ER01</t>
         </is>
       </c>
       <c r="B122" s="5" t="n">
@@ -17338,7 +17344,7 @@
     <row r="123">
       <c r="A123" s="3" t="inlineStr">
         <is>
-          <t>ER02</t>
+          <t>ERGT01</t>
         </is>
       </c>
       <c r="B123" s="5" t="n">
@@ -17384,7 +17390,7 @@
     <row r="124">
       <c r="A124" s="3" t="inlineStr">
         <is>
-          <t>ER01</t>
+          <t>ER02</t>
         </is>
       </c>
       <c r="B124" s="5" t="n">
@@ -17670,7 +17676,7 @@
     <row r="131">
       <c r="A131" s="3" t="inlineStr">
         <is>
-          <t>VP6</t>
+          <t>VP5</t>
         </is>
       </c>
       <c r="B131" s="5" t="n">
@@ -17716,7 +17722,7 @@
     <row r="132">
       <c r="A132" s="3" t="inlineStr">
         <is>
-          <t>VPNL1</t>
+          <t>VP6</t>
         </is>
       </c>
       <c r="B132" s="5" t="n">
@@ -17762,7 +17768,7 @@
     <row r="133">
       <c r="A133" s="3" t="inlineStr">
         <is>
-          <t>VP5</t>
+          <t>VPNL1</t>
         </is>
       </c>
       <c r="B133" s="5" t="n">
@@ -17854,7 +17860,7 @@
     <row r="135">
       <c r="A135" s="3" t="inlineStr">
         <is>
-          <t>TUMT3NL1</t>
+          <t>TUMT3NL2</t>
         </is>
       </c>
       <c r="B135" s="5" t="n">
@@ -17900,7 +17906,7 @@
     <row r="136">
       <c r="A136" s="3" t="inlineStr">
         <is>
-          <t>TUMT3NL2</t>
+          <t>TUMT3NL3</t>
         </is>
       </c>
       <c r="B136" s="5" t="n">
@@ -17946,7 +17952,7 @@
     <row r="137">
       <c r="A137" s="3" t="inlineStr">
         <is>
-          <t>TUMT3NL3</t>
+          <t>TUMT3NL1</t>
         </is>
       </c>
       <c r="B137" s="5" t="n">
@@ -18478,7 +18484,7 @@
     <row r="150">
       <c r="A150" s="3" t="inlineStr">
         <is>
-          <t>WYANGALB</t>
+          <t>WYANGALA</t>
         </is>
       </c>
       <c r="B150" s="5" t="n">
@@ -18524,7 +18530,7 @@
     <row r="151">
       <c r="A151" s="3" t="inlineStr">
         <is>
-          <t>WYANGALA</t>
+          <t>WYANGALB</t>
         </is>
       </c>
       <c r="B151" s="5" t="n">
@@ -18570,7 +18576,7 @@
     <row r="152">
       <c r="A152" s="3" t="inlineStr">
         <is>
-          <t>LUCAS2S2</t>
+          <t>LUCASHGT</t>
         </is>
       </c>
       <c r="B152" s="5" t="n">
@@ -18616,7 +18622,7 @@
     <row r="153">
       <c r="A153" s="3" t="inlineStr">
         <is>
-          <t>LUCASHGT</t>
+          <t>LUCAS2S2</t>
         </is>
       </c>
       <c r="B153" s="5" t="n">
@@ -18938,23 +18944,23 @@
     <row r="160">
       <c r="A160" s="3" t="inlineStr">
         <is>
-          <t>EASTCRK</t>
+          <t>EASTCRK2</t>
         </is>
       </c>
       <c r="B160" s="5" t="n">
-        <v>1.0018</v>
+        <v>1.0021</v>
       </c>
       <c r="C160" s="5" t="n">
-        <v>1.0035</v>
+        <v>1.0021</v>
       </c>
       <c r="D160" s="5" t="n">
-        <v>1.0041</v>
+        <v>1.0021</v>
       </c>
       <c r="E160" s="5" t="n">
-        <v>1.0033</v>
+        <v>1.0021</v>
       </c>
       <c r="F160" s="5" t="n">
-        <v>1.001</v>
+        <v>1.0021</v>
       </c>
       <c r="G160" s="5" t="n">
         <v>1.001</v>
@@ -18984,23 +18990,23 @@
     <row r="161">
       <c r="A161" s="3" t="inlineStr">
         <is>
-          <t>EASTCRK2</t>
+          <t>EASTCRK</t>
         </is>
       </c>
       <c r="B161" s="5" t="n">
-        <v>1.0021</v>
+        <v>1.0018</v>
       </c>
       <c r="C161" s="5" t="n">
-        <v>1.0021</v>
+        <v>1.0035</v>
       </c>
       <c r="D161" s="5" t="n">
-        <v>1.0021</v>
+        <v>1.0041</v>
       </c>
       <c r="E161" s="5" t="n">
-        <v>1.0021</v>
+        <v>1.0033</v>
       </c>
       <c r="F161" s="5" t="n">
-        <v>1.0021</v>
+        <v>1.001</v>
       </c>
       <c r="G161" s="5" t="n">
         <v>1.001</v>
@@ -19140,7 +19146,7 @@
     <row r="165">
       <c r="A165" s="3" t="inlineStr">
         <is>
-          <t>TARALGA1</t>
+          <t>WDLNGN01</t>
         </is>
       </c>
       <c r="B165" s="5" t="n">
@@ -19186,7 +19192,7 @@
     <row r="166">
       <c r="A166" s="3" t="inlineStr">
         <is>
-          <t>WDLNGN01</t>
+          <t>TARALGA1</t>
         </is>
       </c>
       <c r="B166" s="5" t="n">
@@ -19308,7 +19314,7 @@
     <row r="169">
       <c r="A169" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-4</t>
+          <t>TUMUT3-6</t>
         </is>
       </c>
       <c r="B169" s="5" t="n">
@@ -19354,7 +19360,7 @@
     <row r="170">
       <c r="A170" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-3</t>
+          <t>TUMUT3-5</t>
         </is>
       </c>
       <c r="B170" s="5" t="n">
@@ -19400,7 +19406,7 @@
     <row r="171">
       <c r="A171" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-5</t>
+          <t>TUMUT3-4</t>
         </is>
       </c>
       <c r="B171" s="5" t="n">
@@ -19446,7 +19452,7 @@
     <row r="172">
       <c r="A172" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-1</t>
+          <t>TUMUT3-2</t>
         </is>
       </c>
       <c r="B172" s="5" t="n">
@@ -19492,7 +19498,7 @@
     <row r="173">
       <c r="A173" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-2</t>
+          <t>TUMUT3-3</t>
         </is>
       </c>
       <c r="B173" s="5" t="n">
@@ -19538,7 +19544,7 @@
     <row r="174">
       <c r="A174" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-6</t>
+          <t>TUMUT3-1</t>
         </is>
       </c>
       <c r="B174" s="5" t="n">
@@ -19726,29 +19732,29 @@
     <row r="180">
       <c r="A180" s="3" t="inlineStr">
         <is>
-          <t>TERALBA</t>
+          <t>HVGTS</t>
         </is>
       </c>
       <c r="B180" s="5" t="n">
-        <v>0.9926</v>
+        <v>0.974</v>
       </c>
       <c r="C180" s="5" t="n">
-        <v>0.9907</v>
+        <v>0.9679</v>
       </c>
       <c r="D180" s="5" t="n">
-        <v>0.9892</v>
+        <v>0.9582000000000001</v>
       </c>
       <c r="E180" s="5" t="n">
-        <v>0.9901</v>
+        <v>0.9596</v>
       </c>
       <c r="F180" s="5" t="n">
-        <v>0.9903999999999999</v>
+        <v>0.9654</v>
       </c>
       <c r="G180" s="5" t="n">
-        <v>0.9907</v>
+        <v>0.9673</v>
       </c>
       <c r="H180" s="5" t="n">
-        <v>0.9917</v>
+        <v>0.9651999999999999</v>
       </c>
       <c r="I180" s="5" t="inlineStr"/>
       <c r="J180" s="5" t="inlineStr"/>
@@ -19762,7 +19768,7 @@
     <row r="181">
       <c r="A181" s="3" t="inlineStr">
         <is>
-          <t>WOYWOY1</t>
+          <t>KINCUM1</t>
         </is>
       </c>
       <c r="B181" s="5" t="n">
@@ -19798,29 +19804,29 @@
     <row r="182">
       <c r="A182" s="3" t="inlineStr">
         <is>
-          <t>HVGTS</t>
+          <t>AGLNOW1</t>
         </is>
       </c>
       <c r="B182" s="5" t="n">
-        <v>0.974</v>
+        <v>0.9916</v>
       </c>
       <c r="C182" s="5" t="n">
-        <v>0.9679</v>
+        <v>0.9986</v>
       </c>
       <c r="D182" s="5" t="n">
-        <v>0.9582000000000001</v>
+        <v>1.0023</v>
       </c>
       <c r="E182" s="5" t="n">
-        <v>0.9596</v>
+        <v>1.0037</v>
       </c>
       <c r="F182" s="5" t="n">
-        <v>0.9654</v>
+        <v>0.9929</v>
       </c>
       <c r="G182" s="5" t="n">
-        <v>0.9673</v>
+        <v>0.9967</v>
       </c>
       <c r="H182" s="5" t="n">
-        <v>0.9651999999999999</v>
+        <v>0.9929</v>
       </c>
       <c r="I182" s="5" t="inlineStr"/>
       <c r="J182" s="5" t="inlineStr"/>
@@ -19868,29 +19874,29 @@
     <row r="184">
       <c r="A184" s="3" t="inlineStr">
         <is>
-          <t>AGLNOW1</t>
+          <t>LD03</t>
         </is>
       </c>
       <c r="B184" s="5" t="n">
-        <v>0.9916</v>
+        <v>0.9676</v>
       </c>
       <c r="C184" s="5" t="n">
-        <v>0.9986</v>
+        <v>0.9593</v>
       </c>
       <c r="D184" s="5" t="n">
-        <v>1.0023</v>
+        <v>0.9509</v>
       </c>
       <c r="E184" s="5" t="n">
-        <v>1.0037</v>
+        <v>0.9537</v>
       </c>
       <c r="F184" s="5" t="n">
-        <v>0.9929</v>
+        <v>0.9593</v>
       </c>
       <c r="G184" s="5" t="n">
-        <v>0.9967</v>
+        <v>0.9631</v>
       </c>
       <c r="H184" s="5" t="n">
-        <v>0.9929</v>
+        <v>0.9628</v>
       </c>
       <c r="I184" s="5" t="inlineStr"/>
       <c r="J184" s="5" t="inlineStr"/>
@@ -19904,29 +19910,29 @@
     <row r="185">
       <c r="A185" s="3" t="inlineStr">
         <is>
-          <t>KINCUM1</t>
+          <t>TERALBA</t>
         </is>
       </c>
       <c r="B185" s="5" t="n">
-        <v>1.0017</v>
+        <v>0.9926</v>
       </c>
       <c r="C185" s="5" t="n">
-        <v>1.0015</v>
+        <v>0.9907</v>
       </c>
       <c r="D185" s="5" t="n">
-        <v>1.0008</v>
+        <v>0.9892</v>
       </c>
       <c r="E185" s="5" t="n">
-        <v>1.0011</v>
+        <v>0.9901</v>
       </c>
       <c r="F185" s="5" t="n">
-        <v>1.0036</v>
+        <v>0.9903999999999999</v>
       </c>
       <c r="G185" s="5" t="n">
-        <v>1.0019</v>
+        <v>0.9907</v>
       </c>
       <c r="H185" s="5" t="n">
-        <v>1.0037</v>
+        <v>0.9917</v>
       </c>
       <c r="I185" s="5" t="inlineStr"/>
       <c r="J185" s="5" t="inlineStr"/>
@@ -19940,29 +19946,29 @@
     <row r="186">
       <c r="A186" s="3" t="inlineStr">
         <is>
-          <t>LD03</t>
+          <t>WOYWOY1</t>
         </is>
       </c>
       <c r="B186" s="5" t="n">
-        <v>0.9676</v>
+        <v>1.0017</v>
       </c>
       <c r="C186" s="5" t="n">
-        <v>0.9593</v>
+        <v>1.0015</v>
       </c>
       <c r="D186" s="5" t="n">
-        <v>0.9509</v>
+        <v>1.0008</v>
       </c>
       <c r="E186" s="5" t="n">
-        <v>0.9537</v>
+        <v>1.0011</v>
       </c>
       <c r="F186" s="5" t="n">
-        <v>0.9593</v>
+        <v>1.0036</v>
       </c>
       <c r="G186" s="5" t="n">
-        <v>0.9631</v>
+        <v>1.0019</v>
       </c>
       <c r="H186" s="5" t="n">
-        <v>0.9628</v>
+        <v>1.0037</v>
       </c>
       <c r="I186" s="5" t="inlineStr"/>
       <c r="J186" s="5" t="inlineStr"/>
@@ -20014,7 +20020,7 @@
     <row r="188">
       <c r="A188" s="3" t="inlineStr">
         <is>
-          <t>LD02</t>
+          <t>LD01</t>
         </is>
       </c>
       <c r="B188" s="5" t="n">
@@ -20052,7 +20058,7 @@
     <row r="189">
       <c r="A189" s="3" t="inlineStr">
         <is>
-          <t>LD01</t>
+          <t>LD02</t>
         </is>
       </c>
       <c r="B189" s="5" t="n">
@@ -20090,7 +20096,7 @@
     <row r="190">
       <c r="A190" s="3" t="inlineStr">
         <is>
-          <t>WALGRVG1</t>
+          <t>MLLFGEF1</t>
         </is>
       </c>
       <c r="B190" s="5" t="inlineStr"/>
@@ -20100,16 +20106,16 @@
       <c r="F190" s="5" t="inlineStr"/>
       <c r="G190" s="5" t="inlineStr"/>
       <c r="H190" s="5" t="n">
-        <v>1.0011</v>
+        <v>0.9683</v>
       </c>
       <c r="I190" s="5" t="n">
-        <v>1.001</v>
+        <v>0.9687</v>
       </c>
       <c r="J190" s="5" t="n">
-        <v>1.001</v>
+        <v>0.9663</v>
       </c>
       <c r="K190" s="5" t="n">
-        <v>1.001</v>
+        <v>0.9567</v>
       </c>
       <c r="L190" s="5" t="inlineStr"/>
       <c r="M190" s="5" t="inlineStr"/>
@@ -20120,7 +20126,7 @@
     <row r="191">
       <c r="A191" s="3" t="inlineStr">
         <is>
-          <t>MLLFGEF1</t>
+          <t>DPNTBG1</t>
         </is>
       </c>
       <c r="B191" s="5" t="inlineStr"/>
@@ -20129,17 +20135,15 @@
       <c r="E191" s="5" t="inlineStr"/>
       <c r="F191" s="5" t="inlineStr"/>
       <c r="G191" s="5" t="inlineStr"/>
-      <c r="H191" s="5" t="n">
-        <v>0.9683</v>
-      </c>
+      <c r="H191" s="5" t="inlineStr"/>
       <c r="I191" s="5" t="n">
-        <v>0.9687</v>
+        <v>0.9402</v>
       </c>
       <c r="J191" s="5" t="n">
-        <v>0.9663</v>
+        <v>0.9089</v>
       </c>
       <c r="K191" s="5" t="n">
-        <v>0.9567</v>
+        <v>0.9048</v>
       </c>
       <c r="L191" s="5" t="inlineStr"/>
       <c r="M191" s="5" t="inlineStr"/>
@@ -20150,7 +20154,7 @@
     <row r="192">
       <c r="A192" s="3" t="inlineStr">
         <is>
-          <t>BHBG1</t>
+          <t>RESS1G</t>
         </is>
       </c>
       <c r="B192" s="5" t="inlineStr"/>
@@ -20160,12 +20164,14 @@
       <c r="F192" s="5" t="inlineStr"/>
       <c r="G192" s="5" t="inlineStr"/>
       <c r="H192" s="5" t="inlineStr"/>
-      <c r="I192" s="5" t="inlineStr"/>
+      <c r="I192" s="5" t="n">
+        <v>0.9286</v>
+      </c>
       <c r="J192" s="5" t="n">
-        <v>0.8671</v>
+        <v>0.9089</v>
       </c>
       <c r="K192" s="5" t="n">
-        <v>0.8423</v>
+        <v>0.8702</v>
       </c>
       <c r="L192" s="5" t="inlineStr"/>
       <c r="M192" s="5" t="inlineStr"/>
@@ -20176,7 +20182,7 @@
     <row r="193">
       <c r="A193" s="3" t="inlineStr">
         <is>
-          <t>CAPBES1G</t>
+          <t>RIVNBG2</t>
         </is>
       </c>
       <c r="B193" s="5" t="inlineStr"/>
@@ -20186,12 +20192,14 @@
       <c r="F193" s="5" t="inlineStr"/>
       <c r="G193" s="5" t="inlineStr"/>
       <c r="H193" s="5" t="inlineStr"/>
-      <c r="I193" s="5" t="inlineStr"/>
+      <c r="I193" s="5" t="n">
+        <v>0.9058</v>
+      </c>
       <c r="J193" s="5" t="n">
-        <v>0.9704</v>
+        <v>0.9106</v>
       </c>
       <c r="K193" s="5" t="n">
-        <v>0.9337</v>
+        <v>0.9048</v>
       </c>
       <c r="L193" s="5" t="inlineStr"/>
       <c r="M193" s="5" t="inlineStr"/>
@@ -20202,7 +20210,7 @@
     <row r="194">
       <c r="A194" s="3" t="inlineStr">
         <is>
-          <t>QBYNBG1</t>
+          <t>WALGRVG1</t>
         </is>
       </c>
       <c r="B194" s="5" t="inlineStr"/>
@@ -20211,15 +20219,17 @@
       <c r="E194" s="5" t="inlineStr"/>
       <c r="F194" s="5" t="inlineStr"/>
       <c r="G194" s="5" t="inlineStr"/>
-      <c r="H194" s="5" t="inlineStr"/>
+      <c r="H194" s="5" t="n">
+        <v>1.0011</v>
+      </c>
       <c r="I194" s="5" t="n">
-        <v>0.9752</v>
+        <v>1.001</v>
       </c>
       <c r="J194" s="5" t="n">
-        <v>0.979</v>
+        <v>1.001</v>
       </c>
       <c r="K194" s="5" t="n">
-        <v>0.9571</v>
+        <v>1.001</v>
       </c>
       <c r="L194" s="5" t="inlineStr"/>
       <c r="M194" s="5" t="inlineStr"/>
@@ -20230,7 +20240,7 @@
     <row r="195">
       <c r="A195" s="3" t="inlineStr">
         <is>
-          <t>RIVNBG2</t>
+          <t>BHBG1</t>
         </is>
       </c>
       <c r="B195" s="5" t="inlineStr"/>
@@ -20240,14 +20250,12 @@
       <c r="F195" s="5" t="inlineStr"/>
       <c r="G195" s="5" t="inlineStr"/>
       <c r="H195" s="5" t="inlineStr"/>
-      <c r="I195" s="5" t="n">
-        <v>0.9058</v>
-      </c>
+      <c r="I195" s="5" t="inlineStr"/>
       <c r="J195" s="5" t="n">
-        <v>0.9106</v>
+        <v>0.8671</v>
       </c>
       <c r="K195" s="5" t="n">
-        <v>0.9048</v>
+        <v>0.8423</v>
       </c>
       <c r="L195" s="5" t="inlineStr"/>
       <c r="M195" s="5" t="inlineStr"/>
@@ -20258,7 +20266,7 @@
     <row r="196">
       <c r="A196" s="3" t="inlineStr">
         <is>
-          <t>DPNTBG1</t>
+          <t>QBYNBG1</t>
         </is>
       </c>
       <c r="B196" s="5" t="inlineStr"/>
@@ -20269,13 +20277,13 @@
       <c r="G196" s="5" t="inlineStr"/>
       <c r="H196" s="5" t="inlineStr"/>
       <c r="I196" s="5" t="n">
-        <v>0.9402</v>
+        <v>0.9752</v>
       </c>
       <c r="J196" s="5" t="n">
-        <v>0.9089</v>
+        <v>0.979</v>
       </c>
       <c r="K196" s="5" t="n">
-        <v>0.9048</v>
+        <v>0.9571</v>
       </c>
       <c r="L196" s="5" t="inlineStr"/>
       <c r="M196" s="5" t="inlineStr"/>
@@ -20286,7 +20294,7 @@
     <row r="197">
       <c r="A197" s="3" t="inlineStr">
         <is>
-          <t>RESS1G</t>
+          <t>CAPBES1G</t>
         </is>
       </c>
       <c r="B197" s="5" t="inlineStr"/>
@@ -20296,14 +20304,12 @@
       <c r="F197" s="5" t="inlineStr"/>
       <c r="G197" s="5" t="inlineStr"/>
       <c r="H197" s="5" t="inlineStr"/>
-      <c r="I197" s="5" t="n">
-        <v>0.9286</v>
-      </c>
+      <c r="I197" s="5" t="inlineStr"/>
       <c r="J197" s="5" t="n">
-        <v>0.9089</v>
+        <v>0.9704</v>
       </c>
       <c r="K197" s="5" t="n">
-        <v>0.8702</v>
+        <v>0.9337</v>
       </c>
       <c r="L197" s="5" t="inlineStr"/>
       <c r="M197" s="5" t="inlineStr"/>
@@ -20605,7 +20611,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>QPSFB2</t>
+          <t>QPSFB1</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -20615,7 +20621,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Battery</t>
+          <t>Solar</t>
         </is>
       </c>
       <c r="D3" s="5" t="n">
@@ -20634,7 +20640,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>QPSFB1</t>
+          <t>QPSFB2</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -20644,7 +20650,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Solar</t>
+          <t>Battery</t>
         </is>
       </c>
       <c r="D4" s="5" t="n">
@@ -20895,12 +20901,12 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>WYASF1</t>
+          <t>JUNEESF1</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Wyalong Solar Farm</t>
+          <t>Junee Solar Farm</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -20924,12 +20930,12 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>WSTWYSF1</t>
+          <t>SEBSF1</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>West Wyalong Solar Farm</t>
+          <t>Sebastopol Solar Farm</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -20953,12 +20959,12 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>SEBSF1</t>
+          <t>WSTWYSF1</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Sebastopol Solar Farm</t>
+          <t>West Wyalong Solar Farm</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -20982,12 +20988,12 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>JUNEESF1</t>
+          <t>WYASF1</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Junee Solar Farm</t>
+          <t>Wyalong Solar Farm</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -21258,7 +21264,7 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>URANQ11</t>
+          <t>URANQ12</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -21287,7 +21293,7 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>URANQ12</t>
+          <t>URANQ11</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -21664,7 +21670,7 @@
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>TUMT3NL1</t>
+          <t>TUMT3NL2</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -21693,7 +21699,7 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>TUMT3NL2</t>
+          <t>TUMT3NL3</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -21722,7 +21728,7 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>TUMT3NL3</t>
+          <t>TUMT3NL1</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">

</xml_diff>